<commit_message>
[Word] (Selection) Add snippet for getNextRange and getPreviousRange
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/word.xlsx
+++ b/snippet-extractor-metadata/word.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14863876-029E-4319-A045-C665BA386D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23473AC-1060-41C5-AA4D-116ACC111178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2371" uniqueCount="613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2396" uniqueCount="623">
   <si>
     <t>Class</t>
   </si>
@@ -1859,6 +1859,36 @@
   </si>
   <si>
     <t>SelectionInsertFormulaOptions</t>
+  </si>
+  <si>
+    <t>getNextRange</t>
+  </si>
+  <si>
+    <t>getPreviousRange</t>
+  </si>
+  <si>
+    <t>word-selection-get-previous-next-range</t>
+  </si>
+  <si>
+    <t>SelectionNextOptions</t>
+  </si>
+  <si>
+    <t>SelectionPreviousOptions</t>
+  </si>
+  <si>
+    <t>getNextWord</t>
+  </si>
+  <si>
+    <t>getPreviousSentence</t>
+  </si>
+  <si>
+    <t>getPreviousWord</t>
+  </si>
+  <si>
+    <t>getNextParagraph</t>
+  </si>
+  <si>
+    <t>OperationUnit</t>
   </si>
 </sst>
 </file>
@@ -1907,7 +1937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1918,6 +1948,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1973,8 +2004,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F474" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:F474" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F479" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:F479" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{1DA12987-AB2C-4056-A643-B1229DC856C5}" name="Package" dataDxfId="4"/>
     <tableColumn id="1" xr3:uid="{0CD83AD1-F92A-407D-8460-4E881461FD01}" name="Class" dataDxfId="3"/>
@@ -2284,7 +2315,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F474"/>
+  <dimension ref="A1:F479"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="25.08984375" bestFit="1" customWidth="1"/>
@@ -6119,14 +6150,14 @@
       <c r="B210" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C210" s="5" t="s">
+      <c r="C210" s="2" t="s">
         <v>605</v>
       </c>
       <c r="D210" s="2"/>
-      <c r="E210" s="5" t="s">
+      <c r="E210" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="F210" s="5" t="s">
+      <c r="F210" s="2" t="s">
         <v>608</v>
       </c>
     </row>
@@ -7413,20 +7444,21 @@
       </c>
     </row>
     <row r="281" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A281" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B281" s="1" t="s">
-        <v>411</v>
-      </c>
+      <c r="A281" t="s">
+        <v>162</v>
+      </c>
+      <c r="B281" s="4" t="s">
+        <v>622</v>
+      </c>
+      <c r="C281" s="6"/>
       <c r="D281" t="s">
         <v>128</v>
       </c>
-      <c r="E281" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="F281" s="2" t="s">
-        <v>375</v>
+      <c r="E281" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F281" s="5" t="s">
+        <v>618</v>
       </c>
     </row>
     <row r="282" spans="1:6" x14ac:dyDescent="0.35">
@@ -7434,16 +7466,16 @@
         <v>162</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>499</v>
+        <v>411</v>
       </c>
       <c r="D282" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="E282" s="2" t="s">
-        <v>497</v>
+        <v>374</v>
       </c>
       <c r="F282" s="2" t="s">
-        <v>498</v>
+        <v>375</v>
       </c>
     </row>
     <row r="283" spans="1:6" x14ac:dyDescent="0.35">
@@ -7453,11 +7485,8 @@
       <c r="B283" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="C283" t="s">
-        <v>115</v>
-      </c>
-      <c r="D283">
-        <v>1</v>
+      <c r="D283" t="s">
+        <v>144</v>
       </c>
       <c r="E283" s="2" t="s">
         <v>497</v>
@@ -7474,13 +7503,16 @@
         <v>499</v>
       </c>
       <c r="C284" t="s">
-        <v>500</v>
+        <v>115</v>
+      </c>
+      <c r="D284">
+        <v>1</v>
       </c>
       <c r="E284" s="2" t="s">
         <v>497</v>
       </c>
       <c r="F284" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="285" spans="1:6" x14ac:dyDescent="0.35">
@@ -7488,16 +7520,16 @@
         <v>162</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="D285" t="s">
-        <v>144</v>
+        <v>499</v>
+      </c>
+      <c r="C285" t="s">
+        <v>500</v>
       </c>
       <c r="E285" s="2" t="s">
         <v>497</v>
       </c>
       <c r="F285" s="2" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="286" spans="1:6" x14ac:dyDescent="0.35">
@@ -7505,7 +7537,7 @@
         <v>162</v>
       </c>
       <c r="B286" s="1" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="D286" t="s">
         <v>144</v>
@@ -7514,7 +7546,7 @@
         <v>497</v>
       </c>
       <c r="F286" s="2" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
     </row>
     <row r="287" spans="1:6" x14ac:dyDescent="0.35">
@@ -7524,8 +7556,8 @@
       <c r="B287" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="C287" t="s">
-        <v>508</v>
+      <c r="D287" t="s">
+        <v>144</v>
       </c>
       <c r="E287" s="2" t="s">
         <v>497</v>
@@ -7542,13 +7574,13 @@
         <v>504</v>
       </c>
       <c r="C288" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E288" s="2" t="s">
         <v>497</v>
       </c>
       <c r="F288" s="2" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
     </row>
     <row r="289" spans="1:6" x14ac:dyDescent="0.35">
@@ -7556,34 +7588,33 @@
         <v>162</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="D289" t="s">
-        <v>144</v>
+        <v>504</v>
+      </c>
+      <c r="C289" t="s">
+        <v>509</v>
       </c>
       <c r="E289" s="2" t="s">
         <v>497</v>
       </c>
       <c r="F289" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A290" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="D290" t="s">
+        <v>144</v>
+      </c>
+      <c r="E290" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="F290" s="2" t="s">
         <v>527</v>
-      </c>
-    </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A290" t="s">
-        <v>162</v>
-      </c>
-      <c r="B290" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C290" s="2"/>
-      <c r="D290" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E290" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F290" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="291" spans="1:6" x14ac:dyDescent="0.35">
@@ -7593,77 +7624,75 @@
       <c r="B291" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C291" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D291" s="2">
-        <v>1</v>
+      <c r="C291" s="2"/>
+      <c r="D291" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E291" s="1" t="s">
         <v>79</v>
       </c>
       <c r="F291" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="292" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A292" s="1" t="s">
+      <c r="A292" t="s">
         <v>162</v>
       </c>
       <c r="B292" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>360</v>
+        <v>115</v>
       </c>
       <c r="D292" s="2">
         <v>1</v>
       </c>
       <c r="E292" s="1" t="s">
-        <v>350</v>
+        <v>79</v>
       </c>
       <c r="F292" s="2" t="s">
-        <v>360</v>
+        <v>12</v>
       </c>
     </row>
     <row r="293" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A293" t="s">
+      <c r="A293" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B293" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>29</v>
+        <v>360</v>
       </c>
       <c r="D293" s="2">
         <v>1</v>
       </c>
-      <c r="E293" s="2" t="s">
-        <v>75</v>
+      <c r="E293" s="1" t="s">
+        <v>350</v>
       </c>
       <c r="F293" s="2" t="s">
-        <v>28</v>
+        <v>360</v>
       </c>
     </row>
     <row r="294" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A294" s="1" t="s">
+      <c r="A294" t="s">
         <v>162</v>
       </c>
       <c r="B294" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D294" s="2">
         <v>1</v>
       </c>
       <c r="E294" s="2" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="F294" s="2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="295" spans="1:6" x14ac:dyDescent="0.35">
@@ -7674,36 +7703,36 @@
         <v>10</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>556</v>
+        <v>36</v>
       </c>
       <c r="D295" s="2">
         <v>1</v>
       </c>
       <c r="E295" s="2" t="s">
-        <v>570</v>
+        <v>43</v>
       </c>
       <c r="F295" s="2" t="s">
-        <v>151</v>
+        <v>42</v>
       </c>
     </row>
     <row r="296" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A296" t="s">
+      <c r="A296" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B296" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>13</v>
+        <v>556</v>
       </c>
       <c r="D296" s="2">
         <v>1</v>
       </c>
       <c r="E296" s="2" t="s">
-        <v>81</v>
+        <v>570</v>
       </c>
       <c r="F296" s="2" t="s">
-        <v>22</v>
+        <v>151</v>
       </c>
     </row>
     <row r="297" spans="1:6" x14ac:dyDescent="0.35">
@@ -7714,16 +7743,16 @@
         <v>10</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>512</v>
+        <v>13</v>
       </c>
       <c r="D297" s="2">
         <v>1</v>
       </c>
       <c r="E297" s="2" t="s">
-        <v>537</v>
+        <v>81</v>
       </c>
       <c r="F297" s="2" t="s">
-        <v>523</v>
+        <v>22</v>
       </c>
     </row>
     <row r="298" spans="1:6" x14ac:dyDescent="0.35">
@@ -7734,16 +7763,16 @@
         <v>10</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>48</v>
+        <v>512</v>
       </c>
       <c r="D298" s="2">
         <v>1</v>
       </c>
       <c r="E298" s="2" t="s">
-        <v>71</v>
+        <v>537</v>
       </c>
       <c r="F298" s="2" t="s">
-        <v>47</v>
+        <v>523</v>
       </c>
     </row>
     <row r="299" spans="1:6" x14ac:dyDescent="0.35">
@@ -7763,7 +7792,7 @@
         <v>71</v>
       </c>
       <c r="F299" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.35">
@@ -7773,17 +7802,17 @@
       <c r="B300" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C300" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D300" s="1">
+      <c r="C300" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D300" s="2">
         <v>1</v>
       </c>
       <c r="E300" s="2" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="F300" s="2" t="s">
-        <v>7</v>
+        <v>49</v>
       </c>
     </row>
     <row r="301" spans="1:6" x14ac:dyDescent="0.35">
@@ -7793,17 +7822,17 @@
       <c r="B301" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C301" s="2" t="s">
+      <c r="C301" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>1</v>
       </c>
       <c r="E301" s="2" t="s">
         <v>83</v>
       </c>
       <c r="F301" s="2" t="s">
-        <v>66</v>
+        <v>7</v>
       </c>
     </row>
     <row r="302" spans="1:6" x14ac:dyDescent="0.35">
@@ -7814,16 +7843,16 @@
         <v>10</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="D302" s="2">
         <v>1</v>
       </c>
       <c r="E302" s="2" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F302" s="2" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
     </row>
     <row r="303" spans="1:6" x14ac:dyDescent="0.35">
@@ -7834,16 +7863,16 @@
         <v>10</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D303" s="2">
         <v>1</v>
       </c>
       <c r="E303" s="2" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="F303" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="304" spans="1:6" x14ac:dyDescent="0.35">
@@ -7854,14 +7883,16 @@
         <v>10</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D304" s="2"/>
+        <v>59</v>
+      </c>
+      <c r="D304" s="2">
+        <v>1</v>
+      </c>
       <c r="E304" s="2" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="F304" s="2" t="s">
-        <v>18</v>
+        <v>58</v>
       </c>
     </row>
     <row r="305" spans="1:6" x14ac:dyDescent="0.35">
@@ -7872,14 +7903,14 @@
         <v>10</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D305" s="2"/>
       <c r="E305" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F305" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="306" spans="1:6" x14ac:dyDescent="0.35">
@@ -7890,86 +7921,86 @@
         <v>10</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D306" s="2"/>
       <c r="E306" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F306" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="307" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A307" s="1" t="s">
+      <c r="A307" t="s">
         <v>162</v>
       </c>
       <c r="B307" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>379</v>
+        <v>20</v>
       </c>
       <c r="D307" s="2"/>
       <c r="E307" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F307" s="2" t="s">
-        <v>380</v>
+        <v>16</v>
       </c>
     </row>
     <row r="308" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A308" s="3" t="s">
+      <c r="A308" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B308" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D308" s="2"/>
       <c r="E308" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F308" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="309" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A309" t="s">
+      <c r="A309" s="3" t="s">
         <v>162</v>
       </c>
       <c r="B309" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>17</v>
+        <v>381</v>
       </c>
       <c r="D309" s="2"/>
       <c r="E309" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F309" s="2" t="s">
-        <v>17</v>
+        <v>382</v>
       </c>
     </row>
     <row r="310" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A310" s="1" t="s">
+      <c r="A310" t="s">
         <v>162</v>
       </c>
       <c r="B310" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>280</v>
+        <v>17</v>
       </c>
       <c r="D310" s="2"/>
       <c r="E310" s="2" t="s">
-        <v>269</v>
+        <v>80</v>
       </c>
       <c r="F310" s="2" t="s">
-        <v>279</v>
+        <v>17</v>
       </c>
     </row>
     <row r="311" spans="1:6" x14ac:dyDescent="0.35">
@@ -7980,32 +8011,32 @@
         <v>10</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>238</v>
+        <v>280</v>
       </c>
       <c r="D311" s="2"/>
       <c r="E311" s="2" t="s">
-        <v>82</v>
+        <v>269</v>
       </c>
       <c r="F311" s="2" t="s">
-        <v>240</v>
+        <v>279</v>
       </c>
     </row>
     <row r="312" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A312" t="s">
+      <c r="A312" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B312" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>8</v>
+        <v>238</v>
       </c>
       <c r="D312" s="2"/>
-      <c r="E312" s="1" t="s">
-        <v>79</v>
+      <c r="E312" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="F312" s="2" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
     </row>
     <row r="313" spans="1:6" x14ac:dyDescent="0.35">
@@ -8016,14 +8047,14 @@
         <v>10</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>369</v>
+        <v>8</v>
       </c>
       <c r="D313" s="2"/>
       <c r="E313" s="1" t="s">
-        <v>350</v>
+        <v>79</v>
       </c>
       <c r="F313" s="2" t="s">
-        <v>123</v>
+        <v>11</v>
       </c>
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.35">
@@ -8041,25 +8072,25 @@
         <v>350</v>
       </c>
       <c r="F314" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="315" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A315" t="s">
+        <v>162</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C315" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="D315" s="2"/>
+      <c r="E315" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F315" s="2" t="s">
         <v>324</v>
-      </c>
-    </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A315" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B315" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="C315" s="2"/>
-      <c r="D315" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="E315" s="1" t="s">
-        <v>318</v>
-      </c>
-      <c r="F315" s="2" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.35">
@@ -8077,7 +8108,7 @@
         <v>318</v>
       </c>
       <c r="F316" s="2" t="s">
-        <v>319</v>
+        <v>267</v>
       </c>
     </row>
     <row r="317" spans="1:6" x14ac:dyDescent="0.35">
@@ -8085,17 +8116,17 @@
         <v>162</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C317" s="2"/>
       <c r="D317" s="2" t="s">
         <v>345</v>
       </c>
       <c r="E317" s="1" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="F317" s="2" t="s">
-        <v>267</v>
+        <v>319</v>
       </c>
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.35">
@@ -8113,65 +8144,63 @@
         <v>322</v>
       </c>
       <c r="F318" s="2" t="s">
-        <v>324</v>
+        <v>267</v>
       </c>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A319" t="s">
+      <c r="A319" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>190</v>
+        <v>329</v>
       </c>
       <c r="C319" s="2"/>
       <c r="D319" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E319" s="2" t="s">
-        <v>70</v>
+        <v>345</v>
+      </c>
+      <c r="E319" s="1" t="s">
+        <v>322</v>
       </c>
       <c r="F319" s="2" t="s">
-        <v>175</v>
+        <v>324</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A320" s="1" t="s">
+      <c r="A320" t="s">
         <v>162</v>
       </c>
       <c r="B320" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C320" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D320" s="2">
-        <v>1</v>
-      </c>
-      <c r="E320" s="1" t="s">
-        <v>350</v>
+      <c r="C320" s="2"/>
+      <c r="D320" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E320" s="2" t="s">
+        <v>70</v>
       </c>
       <c r="F320" s="2" t="s">
-        <v>353</v>
+        <v>175</v>
       </c>
     </row>
     <row r="321" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A321" t="s">
+      <c r="A321" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B321" s="1" t="s">
         <v>190</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>176</v>
+        <v>100</v>
       </c>
       <c r="D321" s="2">
         <v>1</v>
       </c>
-      <c r="E321" s="2" t="s">
-        <v>70</v>
+      <c r="E321" s="1" t="s">
+        <v>350</v>
       </c>
       <c r="F321" s="2" t="s">
-        <v>175</v>
+        <v>353</v>
       </c>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.35">
@@ -8182,14 +8211,16 @@
         <v>190</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D322" s="2"/>
+        <v>176</v>
+      </c>
+      <c r="D322" s="2">
+        <v>1</v>
+      </c>
       <c r="E322" s="2" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="F322" s="2" t="s">
-        <v>58</v>
+        <v>175</v>
       </c>
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.35">
@@ -8197,17 +8228,17 @@
         <v>162</v>
       </c>
       <c r="B323" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="C323" s="2"/>
-      <c r="D323" s="2" t="s">
-        <v>345</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="C323" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D323" s="2"/>
       <c r="E323" s="2" t="s">
-        <v>323</v>
+        <v>57</v>
       </c>
       <c r="F323" s="2" t="s">
-        <v>267</v>
+        <v>58</v>
       </c>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.35">
@@ -8225,25 +8256,25 @@
         <v>323</v>
       </c>
       <c r="F324" s="2" t="s">
-        <v>325</v>
+        <v>267</v>
       </c>
     </row>
     <row r="325" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A325" s="1" t="s">
+      <c r="A325" t="s">
         <v>162</v>
       </c>
       <c r="B325" s="1" t="s">
-        <v>281</v>
+        <v>346</v>
       </c>
       <c r="C325" s="2"/>
       <c r="D325" s="2" t="s">
-        <v>144</v>
+        <v>345</v>
       </c>
       <c r="E325" s="2" t="s">
-        <v>269</v>
+        <v>323</v>
       </c>
       <c r="F325" s="2" t="s">
-        <v>294</v>
+        <v>325</v>
       </c>
     </row>
     <row r="326" spans="1:6" x14ac:dyDescent="0.35">
@@ -8253,10 +8284,10 @@
       <c r="B326" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="C326" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D326" s="2"/>
+      <c r="C326" s="2"/>
+      <c r="D326" s="2" t="s">
+        <v>144</v>
+      </c>
       <c r="E326" s="2" t="s">
         <v>269</v>
       </c>
@@ -8272,7 +8303,7 @@
         <v>281</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D327" s="2"/>
       <c r="E327" s="2" t="s">
@@ -8287,17 +8318,17 @@
         <v>162</v>
       </c>
       <c r="B328" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C328" s="2"/>
-      <c r="D328" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>281</v>
+      </c>
+      <c r="C328" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D328" s="2"/>
       <c r="E328" s="2" t="s">
-        <v>145</v>
+        <v>269</v>
       </c>
       <c r="F328" s="2" t="s">
-        <v>445</v>
+        <v>294</v>
       </c>
     </row>
     <row r="329" spans="1:6" x14ac:dyDescent="0.35">
@@ -8307,17 +8338,15 @@
       <c r="B329" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C329" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D329" s="2">
-        <v>1</v>
+      <c r="C329" s="2"/>
+      <c r="D329" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E329" s="2" t="s">
-        <v>227</v>
+        <v>145</v>
       </c>
       <c r="F329" s="2" t="s">
-        <v>228</v>
+        <v>445</v>
       </c>
     </row>
     <row r="330" spans="1:6" x14ac:dyDescent="0.35">
@@ -8328,36 +8357,36 @@
         <v>5</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>492</v>
+        <v>229</v>
       </c>
       <c r="D330" s="2">
         <v>1</v>
       </c>
       <c r="E330" s="2" t="s">
-        <v>79</v>
+        <v>227</v>
       </c>
       <c r="F330" s="2" t="s">
-        <v>12</v>
+        <v>228</v>
       </c>
     </row>
     <row r="331" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A331" t="s">
+      <c r="A331" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B331" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C331" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D331" s="1">
+      <c r="C331" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="D331" s="2">
         <v>1</v>
       </c>
       <c r="E331" s="2" t="s">
-        <v>145</v>
+        <v>79</v>
       </c>
       <c r="F331" s="2" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
     </row>
     <row r="332" spans="1:6" x14ac:dyDescent="0.35">
@@ -8368,16 +8397,16 @@
         <v>5</v>
       </c>
       <c r="C332" s="1" t="s">
-        <v>395</v>
+        <v>107</v>
       </c>
       <c r="D332" s="1">
         <v>1</v>
       </c>
       <c r="E332" s="2" t="s">
-        <v>393</v>
+        <v>145</v>
       </c>
       <c r="F332" s="2" t="s">
-        <v>427</v>
+        <v>108</v>
       </c>
     </row>
     <row r="333" spans="1:6" x14ac:dyDescent="0.35">
@@ -8388,16 +8417,16 @@
         <v>5</v>
       </c>
       <c r="C333" s="1" t="s">
-        <v>115</v>
+        <v>395</v>
       </c>
       <c r="D333" s="1">
         <v>1</v>
       </c>
       <c r="E333" s="2" t="s">
-        <v>494</v>
+        <v>393</v>
       </c>
       <c r="F333" s="2" t="s">
-        <v>462</v>
+        <v>427</v>
       </c>
     </row>
     <row r="334" spans="1:6" x14ac:dyDescent="0.35">
@@ -8408,16 +8437,16 @@
         <v>5</v>
       </c>
       <c r="C334" s="1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D334" s="1">
         <v>1</v>
       </c>
       <c r="E334" s="2" t="s">
-        <v>147</v>
+        <v>494</v>
       </c>
       <c r="F334" s="2" t="s">
-        <v>121</v>
+        <v>462</v>
       </c>
     </row>
     <row r="335" spans="1:6" x14ac:dyDescent="0.35">
@@ -8428,16 +8457,16 @@
         <v>5</v>
       </c>
       <c r="C335" s="1" t="s">
-        <v>14</v>
+        <v>121</v>
       </c>
       <c r="D335" s="1">
         <v>1</v>
       </c>
-      <c r="E335" s="1" t="s">
-        <v>79</v>
+      <c r="E335" s="2" t="s">
+        <v>147</v>
       </c>
       <c r="F335" s="2" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
     </row>
     <row r="336" spans="1:6" x14ac:dyDescent="0.35">
@@ -8448,16 +8477,16 @@
         <v>5</v>
       </c>
       <c r="C336" s="1" t="s">
-        <v>106</v>
+        <v>14</v>
       </c>
       <c r="D336" s="1">
         <v>1</v>
       </c>
       <c r="E336" s="1" t="s">
-        <v>145</v>
+        <v>79</v>
       </c>
       <c r="F336" s="2" t="s">
-        <v>106</v>
+        <v>12</v>
       </c>
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.35">
@@ -8468,56 +8497,56 @@
         <v>5</v>
       </c>
       <c r="C337" s="1" t="s">
-        <v>36</v>
+        <v>106</v>
       </c>
       <c r="D337" s="1">
         <v>1</v>
       </c>
-      <c r="E337" s="2" t="s">
-        <v>82</v>
+      <c r="E337" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="F337" s="2" t="s">
-        <v>35</v>
+        <v>106</v>
       </c>
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A338" s="1" t="s">
+      <c r="A338" t="s">
         <v>162</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C338" s="1" t="s">
-        <v>283</v>
+        <v>36</v>
       </c>
       <c r="D338" s="1">
         <v>1</v>
       </c>
       <c r="E338" s="2" t="s">
-        <v>163</v>
+        <v>82</v>
       </c>
       <c r="F338" s="2" t="s">
-        <v>284</v>
+        <v>35</v>
       </c>
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A339" t="s">
+      <c r="A339" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C339" s="1" t="s">
-        <v>88</v>
+        <v>283</v>
       </c>
       <c r="D339" s="1">
         <v>1</v>
       </c>
-      <c r="E339" s="1" t="s">
-        <v>146</v>
+      <c r="E339" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="F339" s="2" t="s">
-        <v>88</v>
+        <v>284</v>
       </c>
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.35">
@@ -8528,16 +8557,16 @@
         <v>5</v>
       </c>
       <c r="C340" s="1" t="s">
-        <v>313</v>
+        <v>88</v>
       </c>
       <c r="D340" s="1">
         <v>1</v>
       </c>
       <c r="E340" s="1" t="s">
-        <v>537</v>
+        <v>146</v>
       </c>
       <c r="F340" s="2" t="s">
-        <v>521</v>
+        <v>88</v>
       </c>
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.35">
@@ -8557,7 +8586,7 @@
         <v>537</v>
       </c>
       <c r="F341" s="2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.35">
@@ -8568,16 +8597,16 @@
         <v>5</v>
       </c>
       <c r="C342" s="1" t="s">
-        <v>556</v>
+        <v>313</v>
       </c>
       <c r="D342" s="1">
         <v>1</v>
       </c>
       <c r="E342" s="1" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F342" s="2" t="s">
-        <v>561</v>
+        <v>524</v>
       </c>
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.35">
@@ -8588,16 +8617,16 @@
         <v>5</v>
       </c>
       <c r="C343" s="1" t="s">
-        <v>512</v>
+        <v>556</v>
       </c>
       <c r="D343" s="1">
         <v>1</v>
       </c>
       <c r="E343" s="1" t="s">
-        <v>537</v>
+        <v>555</v>
       </c>
       <c r="F343" s="2" t="s">
-        <v>511</v>
+        <v>561</v>
       </c>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.35">
@@ -8608,31 +8637,34 @@
         <v>5</v>
       </c>
       <c r="C344" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D344" s="1"/>
+        <v>512</v>
+      </c>
+      <c r="D344" s="1">
+        <v>1</v>
+      </c>
       <c r="E344" s="1" t="s">
-        <v>146</v>
+        <v>537</v>
       </c>
       <c r="F344" s="2" t="s">
-        <v>96</v>
+        <v>511</v>
       </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A345" s="1" t="s">
+      <c r="A345" t="s">
         <v>162</v>
       </c>
       <c r="B345" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C345" t="s">
-        <v>428</v>
-      </c>
-      <c r="E345" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="F345" t="s">
-        <v>422</v>
+      <c r="C345" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D345" s="1"/>
+      <c r="E345" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F345" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.35">
@@ -8642,15 +8674,14 @@
       <c r="B346" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C346" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D346" s="2"/>
+      <c r="C346" t="s">
+        <v>428</v>
+      </c>
       <c r="E346" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F346" s="2" t="s">
-        <v>239</v>
+        <v>393</v>
+      </c>
+      <c r="F346" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="347" spans="1:6" x14ac:dyDescent="0.35">
@@ -8658,53 +8689,53 @@
         <v>162</v>
       </c>
       <c r="B347" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C347" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D347" s="2"/>
+      <c r="E347" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F347" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="348" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A348" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B348" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="C347" s="2"/>
-      <c r="D347" s="2" t="s">
+      <c r="C348" s="2"/>
+      <c r="D348" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E347" s="2" t="s">
+      <c r="E348" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F347" s="2" t="s">
+      <c r="F348" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="348" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A348" t="s">
-        <v>162</v>
-      </c>
-      <c r="B348" s="1" t="s">
+    <row r="349" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A349" t="s">
+        <v>162</v>
+      </c>
+      <c r="B349" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="C348" s="1"/>
-      <c r="D348" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E348" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F348" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="349" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A349" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B349" s="1" t="s">
-        <v>575</v>
       </c>
       <c r="C349" s="1"/>
       <c r="D349" s="1" t="s">
         <v>128</v>
       </c>
       <c r="E349" s="1" t="s">
-        <v>570</v>
+        <v>79</v>
       </c>
       <c r="F349" s="2" t="s">
-        <v>576</v>
+        <v>12</v>
       </c>
     </row>
     <row r="350" spans="1:6" x14ac:dyDescent="0.35">
@@ -8712,7 +8743,7 @@
         <v>162</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C350" s="1"/>
       <c r="D350" s="1" t="s">
@@ -8722,7 +8753,7 @@
         <v>570</v>
       </c>
       <c r="F350" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="351" spans="1:6" x14ac:dyDescent="0.35">
@@ -8730,7 +8761,7 @@
         <v>162</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C351" s="1"/>
       <c r="D351" s="1" t="s">
@@ -8740,7 +8771,7 @@
         <v>570</v>
       </c>
       <c r="F351" s="2" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="352" spans="1:6" x14ac:dyDescent="0.35">
@@ -8748,17 +8779,17 @@
         <v>162</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>418</v>
+        <v>579</v>
       </c>
       <c r="C352" s="1"/>
       <c r="D352" s="1" t="s">
         <v>128</v>
       </c>
       <c r="E352" s="1" t="s">
-        <v>413</v>
+        <v>570</v>
       </c>
       <c r="F352" s="2" t="s">
-        <v>414</v>
+        <v>576</v>
       </c>
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.35">
@@ -8766,37 +8797,35 @@
         <v>162</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>534</v>
+        <v>418</v>
       </c>
       <c r="C353" s="1"/>
       <c r="D353" s="1" t="s">
         <v>128</v>
       </c>
       <c r="E353" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F353" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="354" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A354" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C354" s="1"/>
+      <c r="D354" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E354" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="F353" s="2" t="s">
+      <c r="F354" s="2" t="s">
         <v>533</v>
-      </c>
-    </row>
-    <row r="354" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A354" t="s">
-        <v>162</v>
-      </c>
-      <c r="B354" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C354" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D354" s="2">
-        <v>2</v>
-      </c>
-      <c r="E354" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F354" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="355" spans="1:6" x14ac:dyDescent="0.35">
@@ -8806,17 +8835,17 @@
       <c r="B355" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C355" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D355" s="1">
-        <v>1</v>
+      <c r="C355" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D355" s="2">
+        <v>2</v>
       </c>
       <c r="E355" s="2" t="s">
         <v>78</v>
       </c>
       <c r="F355" s="2" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.35">
@@ -8826,15 +8855,17 @@
       <c r="B356" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C356" s="1"/>
-      <c r="D356" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="E356" s="1" t="s">
-        <v>140</v>
+      <c r="C356" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D356" s="1">
+        <v>1</v>
+      </c>
+      <c r="E356" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="F356" s="2" t="s">
-        <v>141</v>
+        <v>69</v>
       </c>
     </row>
     <row r="357" spans="1:6" x14ac:dyDescent="0.35">
@@ -8842,73 +8873,73 @@
         <v>162</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C357" s="2"/>
-      <c r="D357" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C357" s="1"/>
+      <c r="D357" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E357" s="2" t="s">
+      <c r="E357" s="1" t="s">
         <v>140</v>
       </c>
       <c r="F357" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="358" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
         <v>162</v>
       </c>
-      <c r="B358" s="4" t="s">
-        <v>609</v>
-      </c>
-      <c r="C358" s="5"/>
+      <c r="B358" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C358" s="2"/>
       <c r="D358" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E358" s="5" t="s">
-        <v>606</v>
-      </c>
-      <c r="F358" s="5" t="s">
-        <v>608</v>
+      <c r="E358" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F358" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="359" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
         <v>162</v>
       </c>
-      <c r="B359" s="4" t="s">
+      <c r="B359" s="1" t="s">
         <v>609</v>
       </c>
-      <c r="C359" s="5" t="s">
-        <v>610</v>
-      </c>
-      <c r="D359" s="2">
-        <v>1</v>
-      </c>
-      <c r="E359" s="5" t="s">
+      <c r="C359" s="2"/>
+      <c r="D359" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E359" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="F359" s="5" t="s">
-        <v>607</v>
+      <c r="F359" s="2" t="s">
+        <v>608</v>
       </c>
     </row>
     <row r="360" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
         <v>162</v>
       </c>
-      <c r="B360" s="4" t="s">
-        <v>612</v>
-      </c>
-      <c r="C360" s="5"/>
-      <c r="D360" s="2" t="s">
-        <v>345</v>
+      <c r="B360" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="C360" s="5" t="s">
+        <v>613</v>
+      </c>
+      <c r="D360" s="2">
+        <v>1</v>
       </c>
       <c r="E360" s="5" t="s">
-        <v>606</v>
+        <v>615</v>
       </c>
       <c r="F360" s="5" t="s">
-        <v>611</v>
+        <v>621</v>
       </c>
     </row>
     <row r="361" spans="1:6" x14ac:dyDescent="0.35">
@@ -8916,109 +8947,111 @@
         <v>162</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C361" s="2"/>
-      <c r="D361" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E361" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F361" s="2" t="s">
-        <v>49</v>
+        <v>609</v>
+      </c>
+      <c r="C361" s="5" t="s">
+        <v>614</v>
+      </c>
+      <c r="D361" s="2">
+        <v>1</v>
+      </c>
+      <c r="E361" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F361" s="5" t="s">
+        <v>619</v>
       </c>
     </row>
     <row r="362" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A362" s="1" t="s">
+      <c r="A362" t="s">
         <v>162</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="C362" s="2"/>
-      <c r="D362" s="2" t="s">
-        <v>144</v>
+        <v>609</v>
+      </c>
+      <c r="C362" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="D362" s="2">
+        <v>1</v>
       </c>
       <c r="E362" s="2" t="s">
-        <v>164</v>
+        <v>606</v>
       </c>
       <c r="F362" s="2" t="s">
-        <v>168</v>
+        <v>607</v>
       </c>
     </row>
     <row r="363" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A363" s="1" t="s">
+      <c r="A363" t="s">
         <v>162</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="C363" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="D363" s="2"/>
+        <v>612</v>
+      </c>
+      <c r="C363" s="2"/>
+      <c r="D363" s="2" t="s">
+        <v>345</v>
+      </c>
       <c r="E363" s="2" t="s">
-        <v>164</v>
+        <v>606</v>
       </c>
       <c r="F363" s="2" t="s">
-        <v>168</v>
+        <v>611</v>
       </c>
     </row>
     <row r="364" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B364" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="C364" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="D364" s="2"/>
-      <c r="E364" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="F364" s="2" t="s">
-        <v>168</v>
+      <c r="B364" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="C364" s="5"/>
+      <c r="D364" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="E364" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F364" s="5" t="s">
+        <v>618</v>
       </c>
     </row>
     <row r="365" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B365" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C365" s="2"/>
+      <c r="B365" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="C365" s="5"/>
       <c r="D365" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E365" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="F365" s="2" t="s">
-        <v>166</v>
+        <v>345</v>
+      </c>
+      <c r="E365" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F365" s="5" t="s">
+        <v>620</v>
       </c>
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A366" s="1" t="s">
+      <c r="A366" t="s">
         <v>162</v>
       </c>
       <c r="B366" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C366" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D366" s="2">
-        <v>1</v>
+        <v>159</v>
+      </c>
+      <c r="C366" s="2"/>
+      <c r="D366" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="E366" s="2" t="s">
-        <v>164</v>
+        <v>71</v>
       </c>
       <c r="F366" s="2" t="s">
-        <v>168</v>
+        <v>49</v>
       </c>
     </row>
     <row r="367" spans="1:6" x14ac:dyDescent="0.35">
@@ -9026,17 +9059,17 @@
         <v>162</v>
       </c>
       <c r="B367" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C367" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D367" s="2"/>
+        <v>296</v>
+      </c>
+      <c r="C367" s="2"/>
+      <c r="D367" s="2" t="s">
+        <v>144</v>
+      </c>
       <c r="E367" s="2" t="s">
         <v>164</v>
       </c>
       <c r="F367" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="368" spans="1:6" x14ac:dyDescent="0.35">
@@ -9044,17 +9077,17 @@
         <v>162</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="C368" s="2"/>
-      <c r="D368" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>296</v>
+      </c>
+      <c r="C368" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D368" s="2"/>
       <c r="E368" s="2" t="s">
-        <v>269</v>
+        <v>164</v>
       </c>
       <c r="F368" s="2" t="s">
-        <v>489</v>
+        <v>168</v>
       </c>
     </row>
     <row r="369" spans="1:6" x14ac:dyDescent="0.35">
@@ -9062,17 +9095,17 @@
         <v>162</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="C369" s="2"/>
-      <c r="D369" s="2" t="s">
-        <v>128</v>
-      </c>
+        <v>296</v>
+      </c>
+      <c r="C369" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D369" s="2"/>
       <c r="E369" s="2" t="s">
-        <v>269</v>
+        <v>164</v>
       </c>
       <c r="F369" s="2" t="s">
-        <v>489</v>
+        <v>168</v>
       </c>
     </row>
     <row r="370" spans="1:6" x14ac:dyDescent="0.35">
@@ -9080,17 +9113,17 @@
         <v>162</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>516</v>
+        <v>167</v>
       </c>
       <c r="C370" s="2"/>
       <c r="D370" s="2" t="s">
         <v>144</v>
       </c>
       <c r="E370" s="2" t="s">
-        <v>537</v>
+        <v>164</v>
       </c>
       <c r="F370" s="2" t="s">
-        <v>519</v>
+        <v>166</v>
       </c>
     </row>
     <row r="371" spans="1:6" x14ac:dyDescent="0.35">
@@ -9098,19 +9131,19 @@
         <v>162</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>516</v>
+        <v>167</v>
       </c>
       <c r="C371" s="2" t="s">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="D371" s="2">
         <v>1</v>
       </c>
       <c r="E371" s="2" t="s">
-        <v>537</v>
+        <v>164</v>
       </c>
       <c r="F371" s="2" t="s">
-        <v>522</v>
+        <v>168</v>
       </c>
     </row>
     <row r="372" spans="1:6" x14ac:dyDescent="0.35">
@@ -9118,19 +9151,17 @@
         <v>162</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>516</v>
+        <v>167</v>
       </c>
       <c r="C372" s="2" t="s">
-        <v>583</v>
-      </c>
-      <c r="D372" s="2">
-        <v>1</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="D372" s="2"/>
       <c r="E372" s="2" t="s">
-        <v>570</v>
+        <v>164</v>
       </c>
       <c r="F372" s="2" t="s">
-        <v>584</v>
+        <v>169</v>
       </c>
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.35">
@@ -9138,19 +9169,17 @@
         <v>162</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="C373" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="D373" s="2">
-        <v>1</v>
+        <v>491</v>
+      </c>
+      <c r="C373" s="2"/>
+      <c r="D373" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E373" s="2" t="s">
-        <v>570</v>
+        <v>269</v>
       </c>
       <c r="F373" s="2" t="s">
-        <v>584</v>
+        <v>489</v>
       </c>
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.35">
@@ -9158,19 +9187,17 @@
         <v>162</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="C374" s="2" t="s">
-        <v>587</v>
-      </c>
-      <c r="D374" s="2">
-        <v>1</v>
+        <v>490</v>
+      </c>
+      <c r="C374" s="2"/>
+      <c r="D374" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="E374" s="2" t="s">
-        <v>570</v>
+        <v>269</v>
       </c>
       <c r="F374" s="2" t="s">
-        <v>581</v>
+        <v>489</v>
       </c>
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.35">
@@ -9180,17 +9207,15 @@
       <c r="B375" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="C375" s="2" t="s">
-        <v>588</v>
-      </c>
-      <c r="D375" s="2">
-        <v>1</v>
+      <c r="C375" s="2"/>
+      <c r="D375" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E375" s="2" t="s">
-        <v>570</v>
+        <v>537</v>
       </c>
       <c r="F375" s="2" t="s">
-        <v>581</v>
+        <v>519</v>
       </c>
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.35">
@@ -9201,16 +9226,16 @@
         <v>516</v>
       </c>
       <c r="C376" s="2" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
       <c r="D376" s="2">
         <v>1</v>
       </c>
       <c r="E376" s="2" t="s">
-        <v>570</v>
+        <v>537</v>
       </c>
       <c r="F376" s="2" t="s">
-        <v>571</v>
+        <v>522</v>
       </c>
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.35">
@@ -9221,14 +9246,16 @@
         <v>516</v>
       </c>
       <c r="C377" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="D377" s="2"/>
+        <v>583</v>
+      </c>
+      <c r="D377" s="2">
+        <v>1</v>
+      </c>
       <c r="E377" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F377" s="2" t="s">
-        <v>520</v>
+        <v>584</v>
       </c>
     </row>
     <row r="378" spans="1:6" x14ac:dyDescent="0.35">
@@ -9239,14 +9266,16 @@
         <v>516</v>
       </c>
       <c r="C378" s="2" t="s">
-        <v>597</v>
-      </c>
-      <c r="D378" s="2"/>
+        <v>585</v>
+      </c>
+      <c r="D378" s="2">
+        <v>1</v>
+      </c>
       <c r="E378" s="2" t="s">
-        <v>595</v>
+        <v>570</v>
       </c>
       <c r="F378" s="2" t="s">
-        <v>596</v>
+        <v>584</v>
       </c>
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.35">
@@ -9257,14 +9286,16 @@
         <v>516</v>
       </c>
       <c r="C379" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="D379" s="2"/>
+        <v>587</v>
+      </c>
+      <c r="D379" s="2">
+        <v>1</v>
+      </c>
       <c r="E379" s="2" t="s">
-        <v>555</v>
+        <v>570</v>
       </c>
       <c r="F379" s="2" t="s">
-        <v>564</v>
+        <v>581</v>
       </c>
     </row>
     <row r="380" spans="1:6" x14ac:dyDescent="0.35">
@@ -9275,14 +9306,16 @@
         <v>516</v>
       </c>
       <c r="C380" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="D380" s="2"/>
+        <v>588</v>
+      </c>
+      <c r="D380" s="2">
+        <v>1</v>
+      </c>
       <c r="E380" s="2" t="s">
-        <v>555</v>
+        <v>570</v>
       </c>
       <c r="F380" s="2" t="s">
-        <v>559</v>
+        <v>581</v>
       </c>
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.35">
@@ -9293,14 +9326,16 @@
         <v>516</v>
       </c>
       <c r="C381" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="D381" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="D381" s="2">
+        <v>1</v>
+      </c>
       <c r="E381" s="2" t="s">
         <v>570</v>
       </c>
       <c r="F381" s="2" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
     </row>
     <row r="382" spans="1:6" x14ac:dyDescent="0.35">
@@ -9311,14 +9346,14 @@
         <v>516</v>
       </c>
       <c r="C382" s="2" t="s">
-        <v>589</v>
+        <v>104</v>
       </c>
       <c r="D382" s="2"/>
       <c r="E382" s="2" t="s">
-        <v>570</v>
+        <v>537</v>
       </c>
       <c r="F382" s="2" t="s">
-        <v>576</v>
+        <v>520</v>
       </c>
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.35">
@@ -9329,14 +9364,14 @@
         <v>516</v>
       </c>
       <c r="C383" s="2" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="D383" s="2"/>
       <c r="E383" s="2" t="s">
-        <v>570</v>
+        <v>595</v>
       </c>
       <c r="F383" s="2" t="s">
-        <v>578</v>
+        <v>596</v>
       </c>
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.35">
@@ -9347,14 +9382,14 @@
         <v>516</v>
       </c>
       <c r="C384" s="2" t="s">
-        <v>590</v>
+        <v>563</v>
       </c>
       <c r="D384" s="2"/>
       <c r="E384" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F384" s="2" t="s">
-        <v>576</v>
+        <v>564</v>
       </c>
     </row>
     <row r="385" spans="1:6" x14ac:dyDescent="0.35">
@@ -9365,14 +9400,14 @@
         <v>516</v>
       </c>
       <c r="C385" s="2" t="s">
-        <v>592</v>
+        <v>558</v>
       </c>
       <c r="D385" s="2"/>
       <c r="E385" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F385" s="2" t="s">
-        <v>578</v>
+        <v>559</v>
       </c>
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.35">
@@ -9383,14 +9418,14 @@
         <v>516</v>
       </c>
       <c r="C386" s="2" t="s">
-        <v>586</v>
+        <v>593</v>
       </c>
       <c r="D386" s="2"/>
       <c r="E386" s="2" t="s">
         <v>570</v>
       </c>
       <c r="F386" s="2" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
     </row>
     <row r="387" spans="1:6" x14ac:dyDescent="0.35">
@@ -9401,14 +9436,14 @@
         <v>516</v>
       </c>
       <c r="C387" s="2" t="s">
-        <v>538</v>
+        <v>589</v>
       </c>
       <c r="D387" s="2"/>
       <c r="E387" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F387" s="2" t="s">
-        <v>539</v>
+        <v>576</v>
       </c>
     </row>
     <row r="388" spans="1:6" x14ac:dyDescent="0.35">
@@ -9419,14 +9454,14 @@
         <v>516</v>
       </c>
       <c r="C388" s="2" t="s">
-        <v>541</v>
+        <v>591</v>
       </c>
       <c r="D388" s="2"/>
       <c r="E388" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F388" s="2" t="s">
-        <v>542</v>
+        <v>578</v>
       </c>
     </row>
     <row r="389" spans="1:6" x14ac:dyDescent="0.35">
@@ -9437,14 +9472,14 @@
         <v>516</v>
       </c>
       <c r="C389" s="2" t="s">
-        <v>94</v>
+        <v>590</v>
       </c>
       <c r="D389" s="2"/>
       <c r="E389" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F389" s="2" t="s">
-        <v>514</v>
+        <v>576</v>
       </c>
     </row>
     <row r="390" spans="1:6" x14ac:dyDescent="0.35">
@@ -9452,17 +9487,17 @@
         <v>162</v>
       </c>
       <c r="B390" s="1" t="s">
-        <v>548</v>
-      </c>
-      <c r="C390" s="2"/>
-      <c r="D390" s="2" t="s">
-        <v>128</v>
-      </c>
+        <v>516</v>
+      </c>
+      <c r="C390" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="D390" s="2"/>
       <c r="E390" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F390" s="2" t="s">
-        <v>549</v>
+        <v>578</v>
       </c>
     </row>
     <row r="391" spans="1:6" x14ac:dyDescent="0.35">
@@ -9470,17 +9505,17 @@
         <v>162</v>
       </c>
       <c r="B391" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="C391" s="2"/>
-      <c r="D391" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>516</v>
+      </c>
+      <c r="C391" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="D391" s="2"/>
       <c r="E391" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F391" s="2" t="s">
-        <v>514</v>
+        <v>571</v>
       </c>
     </row>
     <row r="392" spans="1:6" x14ac:dyDescent="0.35">
@@ -9488,19 +9523,17 @@
         <v>162</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C392" s="2" t="s">
-        <v>554</v>
-      </c>
-      <c r="D392" s="2">
-        <v>1</v>
-      </c>
+        <v>538</v>
+      </c>
+      <c r="D392" s="2"/>
       <c r="E392" s="2" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F392" s="2" t="s">
-        <v>562</v>
+        <v>539</v>
       </c>
     </row>
     <row r="393" spans="1:6" x14ac:dyDescent="0.35">
@@ -9508,19 +9541,17 @@
         <v>162</v>
       </c>
       <c r="B393" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C393" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="D393" s="2">
-        <v>1</v>
-      </c>
+        <v>541</v>
+      </c>
+      <c r="D393" s="2"/>
       <c r="E393" s="2" t="s">
         <v>537</v>
       </c>
       <c r="F393" s="2" t="s">
-        <v>519</v>
+        <v>542</v>
       </c>
     </row>
     <row r="394" spans="1:6" x14ac:dyDescent="0.35">
@@ -9528,19 +9559,17 @@
         <v>162</v>
       </c>
       <c r="B394" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C394" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D394" s="2">
-        <v>1</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D394" s="2"/>
       <c r="E394" s="2" t="s">
         <v>537</v>
       </c>
       <c r="F394" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
     </row>
     <row r="395" spans="1:6" x14ac:dyDescent="0.35">
@@ -9548,19 +9577,17 @@
         <v>162</v>
       </c>
       <c r="B395" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="C395" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D395" s="2">
-        <v>1</v>
+        <v>548</v>
+      </c>
+      <c r="C395" s="2"/>
+      <c r="D395" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="E395" s="2" t="s">
         <v>537</v>
       </c>
       <c r="F395" s="2" t="s">
-        <v>536</v>
+        <v>549</v>
       </c>
     </row>
     <row r="396" spans="1:6" x14ac:dyDescent="0.35">
@@ -9570,17 +9597,15 @@
       <c r="B396" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="C396" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="D396" s="2">
-        <v>1</v>
+      <c r="C396" s="2"/>
+      <c r="D396" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E396" s="2" t="s">
-        <v>570</v>
+        <v>537</v>
       </c>
       <c r="F396" s="2" t="s">
-        <v>571</v>
+        <v>514</v>
       </c>
     </row>
     <row r="397" spans="1:6" x14ac:dyDescent="0.35">
@@ -9588,17 +9613,19 @@
         <v>162</v>
       </c>
       <c r="B397" s="1" t="s">
-        <v>565</v>
-      </c>
-      <c r="C397" s="2"/>
-      <c r="D397" s="2" t="s">
-        <v>144</v>
+        <v>513</v>
+      </c>
+      <c r="C397" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="D397" s="2">
+        <v>1</v>
       </c>
       <c r="E397" s="2" t="s">
         <v>555</v>
       </c>
       <c r="F397" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="398" spans="1:6" x14ac:dyDescent="0.35">
@@ -9606,19 +9633,19 @@
         <v>162</v>
       </c>
       <c r="B398" s="1" t="s">
-        <v>565</v>
+        <v>513</v>
       </c>
       <c r="C398" s="2" t="s">
-        <v>301</v>
+        <v>518</v>
       </c>
       <c r="D398" s="2">
         <v>1</v>
       </c>
       <c r="E398" s="2" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F398" s="2" t="s">
-        <v>567</v>
+        <v>519</v>
       </c>
     </row>
     <row r="399" spans="1:6" x14ac:dyDescent="0.35">
@@ -9626,19 +9653,19 @@
         <v>162</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>565</v>
+        <v>513</v>
       </c>
       <c r="C399" s="2" t="s">
-        <v>568</v>
+        <v>100</v>
       </c>
       <c r="D399" s="2">
         <v>1</v>
       </c>
       <c r="E399" s="2" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F399" s="2" t="s">
-        <v>567</v>
+        <v>520</v>
       </c>
     </row>
     <row r="400" spans="1:6" x14ac:dyDescent="0.35">
@@ -9646,17 +9673,19 @@
         <v>162</v>
       </c>
       <c r="B400" s="1" t="s">
-        <v>566</v>
-      </c>
-      <c r="C400" s="2"/>
-      <c r="D400" s="2" t="s">
-        <v>128</v>
+        <v>513</v>
+      </c>
+      <c r="C400" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D400" s="2">
+        <v>1</v>
       </c>
       <c r="E400" s="2" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F400" s="2" t="s">
-        <v>564</v>
+        <v>536</v>
       </c>
     </row>
     <row r="401" spans="1:6" x14ac:dyDescent="0.35">
@@ -9664,11 +9693,13 @@
         <v>162</v>
       </c>
       <c r="B401" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="C401" s="2"/>
-      <c r="D401" s="2" t="s">
-        <v>144</v>
+        <v>513</v>
+      </c>
+      <c r="C401" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="D401" s="2">
+        <v>1</v>
       </c>
       <c r="E401" s="2" t="s">
         <v>570</v>
@@ -9682,19 +9713,17 @@
         <v>162</v>
       </c>
       <c r="B402" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="C402" s="2" t="s">
-        <v>573</v>
-      </c>
-      <c r="D402" s="2">
-        <v>1</v>
+        <v>565</v>
+      </c>
+      <c r="C402" s="2"/>
+      <c r="D402" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E402" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F402" s="2" t="s">
-        <v>574</v>
+        <v>564</v>
       </c>
     </row>
     <row r="403" spans="1:6" x14ac:dyDescent="0.35">
@@ -9702,17 +9731,19 @@
         <v>162</v>
       </c>
       <c r="B403" s="1" t="s">
-        <v>572</v>
+        <v>565</v>
       </c>
       <c r="C403" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="D403" s="2"/>
+        <v>301</v>
+      </c>
+      <c r="D403" s="2">
+        <v>1</v>
+      </c>
       <c r="E403" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F403" s="2" t="s">
-        <v>584</v>
+        <v>567</v>
       </c>
     </row>
     <row r="404" spans="1:6" x14ac:dyDescent="0.35">
@@ -9720,17 +9751,19 @@
         <v>162</v>
       </c>
       <c r="B404" s="1" t="s">
-        <v>580</v>
-      </c>
-      <c r="C404" s="2"/>
-      <c r="D404" s="2" t="s">
-        <v>128</v>
+        <v>565</v>
+      </c>
+      <c r="C404" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="D404" s="2">
+        <v>1</v>
       </c>
       <c r="E404" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F404" s="2" t="s">
-        <v>581</v>
+        <v>567</v>
       </c>
     </row>
     <row r="405" spans="1:6" x14ac:dyDescent="0.35">
@@ -9738,17 +9771,17 @@
         <v>162</v>
       </c>
       <c r="B405" s="1" t="s">
-        <v>582</v>
+        <v>566</v>
       </c>
       <c r="C405" s="2"/>
       <c r="D405" s="2" t="s">
         <v>128</v>
       </c>
       <c r="E405" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F405" s="2" t="s">
-        <v>581</v>
+        <v>564</v>
       </c>
     </row>
     <row r="406" spans="1:6" x14ac:dyDescent="0.35">
@@ -9756,17 +9789,17 @@
         <v>162</v>
       </c>
       <c r="B406" s="1" t="s">
-        <v>550</v>
+        <v>572</v>
       </c>
       <c r="C406" s="2"/>
       <c r="D406" s="2" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E406" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F406" s="2" t="s">
-        <v>549</v>
+        <v>571</v>
       </c>
     </row>
     <row r="407" spans="1:6" x14ac:dyDescent="0.35">
@@ -9774,17 +9807,19 @@
         <v>162</v>
       </c>
       <c r="B407" s="1" t="s">
-        <v>551</v>
-      </c>
-      <c r="C407" s="2"/>
-      <c r="D407" s="2" t="s">
-        <v>128</v>
+        <v>572</v>
+      </c>
+      <c r="C407" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="D407" s="2">
+        <v>1</v>
       </c>
       <c r="E407" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F407" s="2" t="s">
-        <v>549</v>
+        <v>574</v>
       </c>
     </row>
     <row r="408" spans="1:6" x14ac:dyDescent="0.35">
@@ -9792,17 +9827,17 @@
         <v>162</v>
       </c>
       <c r="B408" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="C408" s="2"/>
-      <c r="D408" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>572</v>
+      </c>
+      <c r="C408" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D408" s="2"/>
       <c r="E408" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F408" s="2" t="s">
-        <v>542</v>
+        <v>584</v>
       </c>
     </row>
     <row r="409" spans="1:6" x14ac:dyDescent="0.35">
@@ -9810,17 +9845,17 @@
         <v>162</v>
       </c>
       <c r="B409" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="C409" s="2" t="s">
-        <v>544</v>
-      </c>
-      <c r="D409" s="2"/>
+        <v>580</v>
+      </c>
+      <c r="C409" s="2"/>
+      <c r="D409" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E409" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F409" s="2" t="s">
-        <v>547</v>
+        <v>581</v>
       </c>
     </row>
     <row r="410" spans="1:6" x14ac:dyDescent="0.35">
@@ -9828,17 +9863,17 @@
         <v>162</v>
       </c>
       <c r="B410" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="C410" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D410" s="2"/>
+        <v>582</v>
+      </c>
+      <c r="C410" s="2"/>
+      <c r="D410" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E410" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F410" s="2" t="s">
-        <v>547</v>
+        <v>581</v>
       </c>
     </row>
     <row r="411" spans="1:6" x14ac:dyDescent="0.35">
@@ -9846,7 +9881,7 @@
         <v>162</v>
       </c>
       <c r="B411" s="1" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="C411" s="2"/>
       <c r="D411" s="2" t="s">
@@ -9856,7 +9891,7 @@
         <v>537</v>
       </c>
       <c r="F411" s="2" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="412" spans="1:6" x14ac:dyDescent="0.35">
@@ -9864,7 +9899,7 @@
         <v>162</v>
       </c>
       <c r="B412" s="1" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="C412" s="2"/>
       <c r="D412" s="2" t="s">
@@ -9874,7 +9909,7 @@
         <v>537</v>
       </c>
       <c r="F412" s="2" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="413" spans="1:6" x14ac:dyDescent="0.35">
@@ -9882,17 +9917,17 @@
         <v>162</v>
       </c>
       <c r="B413" s="1" t="s">
-        <v>517</v>
+        <v>543</v>
       </c>
       <c r="C413" s="2"/>
       <c r="D413" s="2" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E413" s="2" t="s">
         <v>537</v>
       </c>
       <c r="F413" s="2" t="s">
-        <v>514</v>
+        <v>542</v>
       </c>
     </row>
     <row r="414" spans="1:6" x14ac:dyDescent="0.35">
@@ -9900,17 +9935,17 @@
         <v>162</v>
       </c>
       <c r="B414" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C414" s="2"/>
-      <c r="D414" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>543</v>
+      </c>
+      <c r="C414" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="D414" s="2"/>
       <c r="E414" s="2" t="s">
-        <v>269</v>
+        <v>537</v>
       </c>
       <c r="F414" s="2" t="s">
-        <v>279</v>
+        <v>547</v>
       </c>
     </row>
     <row r="415" spans="1:6" x14ac:dyDescent="0.35">
@@ -9918,19 +9953,17 @@
         <v>162</v>
       </c>
       <c r="B415" s="1" t="s">
-        <v>275</v>
+        <v>543</v>
       </c>
       <c r="C415" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D415" s="2">
-        <v>1</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D415" s="2"/>
       <c r="E415" s="2" t="s">
-        <v>269</v>
+        <v>537</v>
       </c>
       <c r="F415" s="2" t="s">
-        <v>282</v>
+        <v>547</v>
       </c>
     </row>
     <row r="416" spans="1:6" x14ac:dyDescent="0.35">
@@ -9938,17 +9971,17 @@
         <v>162</v>
       </c>
       <c r="B416" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C416" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="D416" s="2"/>
+        <v>545</v>
+      </c>
+      <c r="C416" s="2"/>
+      <c r="D416" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E416" s="2" t="s">
-        <v>269</v>
+        <v>537</v>
       </c>
       <c r="F416" s="2" t="s">
-        <v>378</v>
+        <v>547</v>
       </c>
     </row>
     <row r="417" spans="1:6" x14ac:dyDescent="0.35">
@@ -9956,17 +9989,17 @@
         <v>162</v>
       </c>
       <c r="B417" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C417" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="D417" s="2"/>
+        <v>546</v>
+      </c>
+      <c r="C417" s="2"/>
+      <c r="D417" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E417" s="2" t="s">
-        <v>269</v>
+        <v>537</v>
       </c>
       <c r="F417" s="2" t="s">
-        <v>295</v>
+        <v>547</v>
       </c>
     </row>
     <row r="418" spans="1:6" x14ac:dyDescent="0.35">
@@ -9974,17 +10007,17 @@
         <v>162</v>
       </c>
       <c r="B418" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C418" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="D418" s="2"/>
+        <v>517</v>
+      </c>
+      <c r="C418" s="2"/>
+      <c r="D418" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E418" s="2" t="s">
-        <v>481</v>
+        <v>537</v>
       </c>
       <c r="F418" s="2" t="s">
-        <v>64</v>
+        <v>514</v>
       </c>
     </row>
     <row r="419" spans="1:6" x14ac:dyDescent="0.35">
@@ -9994,10 +10027,10 @@
       <c r="B419" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="C419" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="D419" s="2"/>
+      <c r="C419" s="2"/>
+      <c r="D419" s="2" t="s">
+        <v>144</v>
+      </c>
       <c r="E419" s="2" t="s">
         <v>269</v>
       </c>
@@ -10013,14 +10046,16 @@
         <v>275</v>
       </c>
       <c r="C420" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="D420" s="2"/>
+        <v>97</v>
+      </c>
+      <c r="D420" s="2">
+        <v>1</v>
+      </c>
       <c r="E420" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F420" s="2" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
     </row>
     <row r="421" spans="1:6" x14ac:dyDescent="0.35">
@@ -10031,14 +10066,14 @@
         <v>275</v>
       </c>
       <c r="C421" s="2" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D421" s="2"/>
       <c r="E421" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F421" s="2" t="s">
-        <v>489</v>
+        <v>378</v>
       </c>
     </row>
     <row r="422" spans="1:6" x14ac:dyDescent="0.35">
@@ -10046,17 +10081,17 @@
         <v>162</v>
       </c>
       <c r="B422" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="C422" s="2"/>
-      <c r="D422" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="C422" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D422" s="2"/>
       <c r="E422" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F422" s="2" t="s">
-        <v>270</v>
+        <v>295</v>
       </c>
     </row>
     <row r="423" spans="1:6" x14ac:dyDescent="0.35">
@@ -10064,19 +10099,17 @@
         <v>162</v>
       </c>
       <c r="B423" s="1" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="D423" s="2">
-        <v>1</v>
-      </c>
+        <v>486</v>
+      </c>
+      <c r="D423" s="2"/>
       <c r="E423" s="2" t="s">
-        <v>269</v>
+        <v>481</v>
       </c>
       <c r="F423" s="2" t="s">
-        <v>273</v>
+        <v>64</v>
       </c>
     </row>
     <row r="424" spans="1:6" x14ac:dyDescent="0.35">
@@ -10084,19 +10117,17 @@
         <v>162</v>
       </c>
       <c r="B424" s="1" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C424" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="D424" s="2">
-        <v>1</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="D424" s="2"/>
       <c r="E424" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F424" s="2" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
     </row>
     <row r="425" spans="1:6" x14ac:dyDescent="0.35">
@@ -10104,17 +10135,17 @@
         <v>162</v>
       </c>
       <c r="B425" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="C425" s="2"/>
-      <c r="D425" s="2" t="s">
-        <v>128</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="C425" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D425" s="2"/>
       <c r="E425" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F425" s="2" t="s">
-        <v>279</v>
+        <v>294</v>
       </c>
     </row>
     <row r="426" spans="1:6" x14ac:dyDescent="0.35">
@@ -10122,39 +10153,35 @@
         <v>162</v>
       </c>
       <c r="B426" s="1" t="s">
-        <v>56</v>
+        <v>275</v>
       </c>
       <c r="C426" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D426" s="2">
-        <v>1</v>
-      </c>
+        <v>488</v>
+      </c>
+      <c r="D426" s="2"/>
       <c r="E426" s="2" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="F426" s="2" t="s">
-        <v>198</v>
+        <v>489</v>
       </c>
     </row>
     <row r="427" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A427" t="s">
+      <c r="A427" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B427" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C427" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D427" s="1">
-        <v>1</v>
+        <v>271</v>
+      </c>
+      <c r="C427" s="2"/>
+      <c r="D427" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E427" s="2" t="s">
-        <v>52</v>
+        <v>269</v>
       </c>
       <c r="F427" s="2" t="s">
-        <v>54</v>
+        <v>270</v>
       </c>
     </row>
     <row r="428" spans="1:6" x14ac:dyDescent="0.35">
@@ -10162,19 +10189,19 @@
         <v>162</v>
       </c>
       <c r="B428" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C428" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="D428" s="1">
+        <v>271</v>
+      </c>
+      <c r="C428" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D428" s="2">
         <v>1</v>
       </c>
       <c r="E428" s="2" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="F428" s="2" t="s">
-        <v>203</v>
+        <v>273</v>
       </c>
     </row>
     <row r="429" spans="1:6" x14ac:dyDescent="0.35">
@@ -10182,17 +10209,19 @@
         <v>162</v>
       </c>
       <c r="B429" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C429" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D429" s="1"/>
+        <v>271</v>
+      </c>
+      <c r="C429" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D429" s="2">
+        <v>1</v>
+      </c>
       <c r="E429" s="2" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="F429" s="2" t="s">
-        <v>194</v>
+        <v>270</v>
       </c>
     </row>
     <row r="430" spans="1:6" x14ac:dyDescent="0.35">
@@ -10200,17 +10229,17 @@
         <v>162</v>
       </c>
       <c r="B430" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C430" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="D430" s="1"/>
+        <v>274</v>
+      </c>
+      <c r="C430" s="2"/>
+      <c r="D430" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E430" s="2" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="F430" s="2" t="s">
-        <v>194</v>
+        <v>279</v>
       </c>
     </row>
     <row r="431" spans="1:6" x14ac:dyDescent="0.35">
@@ -10220,33 +10249,37 @@
       <c r="B431" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C431" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D431" s="1"/>
+      <c r="C431" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D431" s="2">
+        <v>1</v>
+      </c>
       <c r="E431" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F431" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="432" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A432" s="1" t="s">
+      <c r="A432" t="s">
         <v>162</v>
       </c>
       <c r="B432" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C432" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="D432" s="1"/>
+        <v>55</v>
+      </c>
+      <c r="D432" s="1">
+        <v>1</v>
+      </c>
       <c r="E432" s="2" t="s">
-        <v>193</v>
+        <v>52</v>
       </c>
       <c r="F432" s="2" t="s">
-        <v>194</v>
+        <v>54</v>
       </c>
     </row>
     <row r="433" spans="1:6" x14ac:dyDescent="0.35">
@@ -10256,15 +10289,17 @@
       <c r="B433" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C433" s="2"/>
-      <c r="D433" s="2" t="s">
-        <v>144</v>
+      <c r="C433" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="D433" s="1">
+        <v>1</v>
       </c>
       <c r="E433" s="2" t="s">
-        <v>52</v>
+        <v>193</v>
       </c>
       <c r="F433" s="2" t="s">
-        <v>53</v>
+        <v>203</v>
       </c>
     </row>
     <row r="434" spans="1:6" x14ac:dyDescent="0.35">
@@ -10272,16 +10307,17 @@
         <v>162</v>
       </c>
       <c r="B434" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D434" t="s">
-        <v>144</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C434" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D434" s="1"/>
       <c r="E434" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F434" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="435" spans="1:6" x14ac:dyDescent="0.35">
@@ -10289,16 +10325,17 @@
         <v>162</v>
       </c>
       <c r="B435" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C435" t="s">
-        <v>200</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C435" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D435" s="1"/>
       <c r="E435" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F435" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="436" spans="1:6" x14ac:dyDescent="0.35">
@@ -10306,16 +10343,17 @@
         <v>162</v>
       </c>
       <c r="B436" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C436" t="s">
-        <v>94</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C436" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D436" s="1"/>
       <c r="E436" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F436" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="437" spans="1:6" x14ac:dyDescent="0.35">
@@ -10323,33 +10361,35 @@
         <v>162</v>
       </c>
       <c r="B437" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C437" t="s">
-        <v>201</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C437" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="D437" s="1"/>
       <c r="E437" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F437" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="438" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A438" t="s">
-        <v>162</v>
-      </c>
-      <c r="B438" t="s">
-        <v>148</v>
-      </c>
-      <c r="D438" t="s">
+      <c r="A438" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B438" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C438" s="2"/>
+      <c r="D438" s="2" t="s">
         <v>144</v>
       </c>
       <c r="E438" s="2" t="s">
-        <v>193</v>
+        <v>52</v>
       </c>
       <c r="F438" s="2" t="s">
-        <v>212</v>
+        <v>53</v>
       </c>
     </row>
     <row r="439" spans="1:6" x14ac:dyDescent="0.35">
@@ -10357,19 +10397,16 @@
         <v>162</v>
       </c>
       <c r="B439" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="C439" t="s">
-        <v>199</v>
-      </c>
-      <c r="D439">
-        <v>2</v>
+        <v>210</v>
+      </c>
+      <c r="D439" t="s">
+        <v>144</v>
       </c>
       <c r="E439" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F439" s="2" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
     </row>
     <row r="440" spans="1:6" x14ac:dyDescent="0.35">
@@ -10377,61 +10414,58 @@
         <v>162</v>
       </c>
       <c r="B440" s="1" t="s">
-        <v>148</v>
+        <v>210</v>
       </c>
       <c r="C440" t="s">
-        <v>204</v>
-      </c>
-      <c r="D440">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="E440" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F440" s="2" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
     </row>
     <row r="441" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A441" t="s">
-        <v>162</v>
-      </c>
-      <c r="B441" t="s">
-        <v>148</v>
+      <c r="A441" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B441" s="1" t="s">
+        <v>210</v>
       </c>
       <c r="C441" t="s">
-        <v>195</v>
+        <v>94</v>
       </c>
       <c r="E441" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F441" s="2" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
     </row>
     <row r="442" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A442" t="s">
-        <v>162</v>
-      </c>
-      <c r="B442" t="s">
-        <v>148</v>
+      <c r="A442" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B442" s="1" t="s">
+        <v>210</v>
       </c>
       <c r="C442" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E442" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F442" s="2" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
     </row>
     <row r="443" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A443" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B443" s="1" t="s">
-        <v>450</v>
+      <c r="A443" t="s">
+        <v>162</v>
+      </c>
+      <c r="B443" t="s">
+        <v>148</v>
       </c>
       <c r="D443" t="s">
         <v>144</v>
@@ -10448,16 +10482,19 @@
         <v>162</v>
       </c>
       <c r="B444" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="D444" t="s">
-        <v>144</v>
+        <v>148</v>
+      </c>
+      <c r="C444" t="s">
+        <v>199</v>
+      </c>
+      <c r="D444">
+        <v>2</v>
       </c>
       <c r="E444" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F444" s="2" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
     </row>
     <row r="445" spans="1:6" x14ac:dyDescent="0.35">
@@ -10465,30 +10502,30 @@
         <v>162</v>
       </c>
       <c r="B445" s="1" t="s">
-        <v>192</v>
+        <v>148</v>
       </c>
       <c r="C445" t="s">
-        <v>100</v>
+        <v>204</v>
       </c>
       <c r="D445">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E445" s="2" t="s">
-        <v>52</v>
+        <v>193</v>
       </c>
       <c r="F445" s="2" t="s">
-        <v>54</v>
+        <v>214</v>
       </c>
     </row>
     <row r="446" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A446" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B446" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="D446" t="s">
-        <v>144</v>
+      <c r="A446" t="s">
+        <v>162</v>
+      </c>
+      <c r="B446" t="s">
+        <v>148</v>
+      </c>
+      <c r="C446" t="s">
+        <v>195</v>
       </c>
       <c r="E446" s="2" t="s">
         <v>193</v>
@@ -10498,23 +10535,20 @@
       </c>
     </row>
     <row r="447" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A447" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B447" s="1" t="s">
-        <v>209</v>
+      <c r="A447" t="s">
+        <v>162</v>
+      </c>
+      <c r="B447" t="s">
+        <v>148</v>
       </c>
       <c r="C447" t="s">
-        <v>199</v>
-      </c>
-      <c r="D447">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="E447" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F447" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="448" spans="1:6" x14ac:dyDescent="0.35">
@@ -10522,19 +10556,16 @@
         <v>162</v>
       </c>
       <c r="B448" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C448" t="s">
-        <v>204</v>
-      </c>
-      <c r="D448">
-        <v>1</v>
+        <v>450</v>
+      </c>
+      <c r="D448" t="s">
+        <v>144</v>
       </c>
       <c r="E448" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F448" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="449" spans="1:6" x14ac:dyDescent="0.35">
@@ -10542,16 +10573,16 @@
         <v>162</v>
       </c>
       <c r="B449" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C449" t="s">
-        <v>449</v>
+        <v>192</v>
+      </c>
+      <c r="D449" t="s">
+        <v>144</v>
       </c>
       <c r="E449" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F449" s="2" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
     </row>
     <row r="450" spans="1:6" x14ac:dyDescent="0.35">
@@ -10559,16 +10590,19 @@
         <v>162</v>
       </c>
       <c r="B450" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="D450" t="s">
-        <v>144</v>
-      </c>
-      <c r="E450" t="s">
-        <v>193</v>
-      </c>
-      <c r="F450" t="s">
-        <v>206</v>
+        <v>192</v>
+      </c>
+      <c r="C450" t="s">
+        <v>100</v>
+      </c>
+      <c r="D450">
+        <v>1</v>
+      </c>
+      <c r="E450" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F450" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.35">
@@ -10576,19 +10610,16 @@
         <v>162</v>
       </c>
       <c r="B451" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="C451" t="s">
-        <v>100</v>
-      </c>
-      <c r="D451">
-        <v>1</v>
-      </c>
-      <c r="E451" t="s">
+        <v>209</v>
+      </c>
+      <c r="D451" t="s">
+        <v>144</v>
+      </c>
+      <c r="E451" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="F451" t="s">
-        <v>208</v>
+      <c r="F451" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="452" spans="1:6" x14ac:dyDescent="0.35">
@@ -10596,16 +10627,19 @@
         <v>162</v>
       </c>
       <c r="B452" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="D452" t="s">
-        <v>144</v>
-      </c>
-      <c r="E452" t="s">
-        <v>374</v>
-      </c>
-      <c r="F452" t="s">
-        <v>376</v>
+        <v>209</v>
+      </c>
+      <c r="C452" t="s">
+        <v>199</v>
+      </c>
+      <c r="D452">
+        <v>1</v>
+      </c>
+      <c r="E452" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F452" s="2" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="453" spans="1:6" x14ac:dyDescent="0.35">
@@ -10613,16 +10647,19 @@
         <v>162</v>
       </c>
       <c r="B453" s="1" t="s">
-        <v>540</v>
-      </c>
-      <c r="D453" t="s">
-        <v>144</v>
-      </c>
-      <c r="E453" t="s">
-        <v>537</v>
-      </c>
-      <c r="F453" t="s">
-        <v>539</v>
+        <v>209</v>
+      </c>
+      <c r="C453" t="s">
+        <v>204</v>
+      </c>
+      <c r="D453">
+        <v>1</v>
+      </c>
+      <c r="E453" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F453" s="2" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="454" spans="1:6" x14ac:dyDescent="0.35">
@@ -10630,16 +10667,16 @@
         <v>162</v>
       </c>
       <c r="B454" s="1" t="s">
-        <v>540</v>
+        <v>209</v>
       </c>
       <c r="C454" t="s">
-        <v>552</v>
-      </c>
-      <c r="E454" t="s">
-        <v>537</v>
-      </c>
-      <c r="F454" t="s">
-        <v>549</v>
+        <v>449</v>
+      </c>
+      <c r="E454" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F454" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="455" spans="1:6" x14ac:dyDescent="0.35">
@@ -10647,16 +10684,16 @@
         <v>162</v>
       </c>
       <c r="B455" s="1" t="s">
-        <v>540</v>
-      </c>
-      <c r="C455" t="s">
-        <v>553</v>
+        <v>207</v>
+      </c>
+      <c r="D455" t="s">
+        <v>144</v>
       </c>
       <c r="E455" t="s">
-        <v>537</v>
+        <v>193</v>
       </c>
       <c r="F455" t="s">
-        <v>549</v>
+        <v>206</v>
       </c>
     </row>
     <row r="456" spans="1:6" x14ac:dyDescent="0.35">
@@ -10664,16 +10701,19 @@
         <v>162</v>
       </c>
       <c r="B456" s="1" t="s">
-        <v>540</v>
+        <v>207</v>
       </c>
       <c r="C456" t="s">
-        <v>196</v>
+        <v>100</v>
+      </c>
+      <c r="D456">
+        <v>1</v>
       </c>
       <c r="E456" t="s">
-        <v>537</v>
+        <v>193</v>
       </c>
       <c r="F456" t="s">
-        <v>549</v>
+        <v>208</v>
       </c>
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.35">
@@ -10681,16 +10721,16 @@
         <v>162</v>
       </c>
       <c r="B457" s="1" t="s">
-        <v>335</v>
+        <v>373</v>
       </c>
       <c r="D457" t="s">
         <v>144</v>
       </c>
       <c r="E457" t="s">
-        <v>331</v>
+        <v>374</v>
       </c>
       <c r="F457" t="s">
-        <v>344</v>
+        <v>376</v>
       </c>
     </row>
     <row r="458" spans="1:6" x14ac:dyDescent="0.35">
@@ -10698,19 +10738,16 @@
         <v>162</v>
       </c>
       <c r="B458" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="C458" t="s">
-        <v>336</v>
-      </c>
-      <c r="D458">
-        <v>1</v>
+        <v>540</v>
+      </c>
+      <c r="D458" t="s">
+        <v>144</v>
       </c>
       <c r="E458" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="F458" t="s">
-        <v>337</v>
+        <v>539</v>
       </c>
     </row>
     <row r="459" spans="1:6" x14ac:dyDescent="0.35">
@@ -10718,19 +10755,16 @@
         <v>162</v>
       </c>
       <c r="B459" s="1" t="s">
-        <v>335</v>
+        <v>540</v>
       </c>
       <c r="C459" t="s">
-        <v>102</v>
-      </c>
-      <c r="D459">
-        <v>1</v>
+        <v>552</v>
       </c>
       <c r="E459" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="F459" t="s">
-        <v>344</v>
+        <v>549</v>
       </c>
     </row>
     <row r="460" spans="1:6" x14ac:dyDescent="0.35">
@@ -10738,19 +10772,16 @@
         <v>162</v>
       </c>
       <c r="B460" s="1" t="s">
-        <v>335</v>
+        <v>540</v>
       </c>
       <c r="C460" t="s">
-        <v>115</v>
-      </c>
-      <c r="D460">
-        <v>1</v>
+        <v>553</v>
       </c>
       <c r="E460" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="F460" t="s">
-        <v>334</v>
+        <v>549</v>
       </c>
     </row>
     <row r="461" spans="1:6" x14ac:dyDescent="0.35">
@@ -10758,19 +10789,16 @@
         <v>162</v>
       </c>
       <c r="B461" s="1" t="s">
-        <v>335</v>
+        <v>540</v>
       </c>
       <c r="C461" t="s">
-        <v>338</v>
-      </c>
-      <c r="D461">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="E461" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="F461" t="s">
-        <v>339</v>
+        <v>549</v>
       </c>
     </row>
     <row r="462" spans="1:6" x14ac:dyDescent="0.35">
@@ -10778,7 +10806,7 @@
         <v>162</v>
       </c>
       <c r="B462" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D462" t="s">
         <v>144</v>
@@ -10787,7 +10815,7 @@
         <v>331</v>
       </c>
       <c r="F462" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
     </row>
     <row r="463" spans="1:6" x14ac:dyDescent="0.35">
@@ -10795,10 +10823,10 @@
         <v>162</v>
       </c>
       <c r="B463" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C463" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="D463">
         <v>1</v>
@@ -10807,7 +10835,7 @@
         <v>331</v>
       </c>
       <c r="F463" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
     </row>
     <row r="464" spans="1:6" x14ac:dyDescent="0.35">
@@ -10815,10 +10843,10 @@
         <v>162</v>
       </c>
       <c r="B464" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C464" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D464">
         <v>1</v>
@@ -10827,7 +10855,7 @@
         <v>331</v>
       </c>
       <c r="F464" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
     </row>
     <row r="465" spans="1:6" x14ac:dyDescent="0.35">
@@ -10835,10 +10863,10 @@
         <v>162</v>
       </c>
       <c r="B465" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C465" t="s">
-        <v>342</v>
+        <v>115</v>
       </c>
       <c r="D465">
         <v>1</v>
@@ -10847,7 +10875,7 @@
         <v>331</v>
       </c>
       <c r="F465" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.35">
@@ -10855,16 +10883,19 @@
         <v>162</v>
       </c>
       <c r="B466" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="D466" t="s">
-        <v>128</v>
+        <v>335</v>
+      </c>
+      <c r="C466" t="s">
+        <v>338</v>
+      </c>
+      <c r="D466">
+        <v>1</v>
       </c>
       <c r="E466" t="s">
         <v>331</v>
       </c>
       <c r="F466" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.35">
@@ -10872,16 +10903,16 @@
         <v>162</v>
       </c>
       <c r="B467" s="1" t="s">
-        <v>482</v>
+        <v>333</v>
       </c>
       <c r="D467" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E467" t="s">
-        <v>481</v>
+        <v>331</v>
       </c>
       <c r="F467" t="s">
-        <v>64</v>
+        <v>334</v>
       </c>
     </row>
     <row r="468" spans="1:6" x14ac:dyDescent="0.35">
@@ -10889,16 +10920,19 @@
         <v>162</v>
       </c>
       <c r="B468" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="D468" t="s">
-        <v>128</v>
+        <v>333</v>
+      </c>
+      <c r="C468" t="s">
+        <v>340</v>
+      </c>
+      <c r="D468">
+        <v>1</v>
       </c>
       <c r="E468" t="s">
-        <v>193</v>
+        <v>331</v>
       </c>
       <c r="F468" t="s">
-        <v>206</v>
+        <v>341</v>
       </c>
     </row>
     <row r="469" spans="1:6" x14ac:dyDescent="0.35">
@@ -10906,16 +10940,19 @@
         <v>162</v>
       </c>
       <c r="B469" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="D469" t="s">
-        <v>144</v>
+        <v>333</v>
+      </c>
+      <c r="C469" t="s">
+        <v>100</v>
+      </c>
+      <c r="D469">
+        <v>1</v>
       </c>
       <c r="E469" t="s">
-        <v>497</v>
+        <v>331</v>
       </c>
       <c r="F469" t="s">
-        <v>503</v>
+        <v>334</v>
       </c>
     </row>
     <row r="470" spans="1:6" x14ac:dyDescent="0.35">
@@ -10923,19 +10960,19 @@
         <v>162</v>
       </c>
       <c r="B470" s="1" t="s">
-        <v>502</v>
+        <v>333</v>
       </c>
       <c r="C470" t="s">
-        <v>415</v>
+        <v>342</v>
       </c>
       <c r="D470">
         <v>1</v>
       </c>
       <c r="E470" t="s">
-        <v>532</v>
+        <v>331</v>
       </c>
       <c r="F470" t="s">
-        <v>533</v>
+        <v>343</v>
       </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.35">
@@ -10943,16 +10980,16 @@
         <v>162</v>
       </c>
       <c r="B471" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="C471" t="s">
-        <v>506</v>
+        <v>442</v>
+      </c>
+      <c r="D471" t="s">
+        <v>128</v>
       </c>
       <c r="E471" t="s">
-        <v>497</v>
+        <v>331</v>
       </c>
       <c r="F471" t="s">
-        <v>507</v>
+        <v>344</v>
       </c>
     </row>
     <row r="472" spans="1:6" x14ac:dyDescent="0.35">
@@ -10960,16 +10997,16 @@
         <v>162</v>
       </c>
       <c r="B472" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="C472" t="s">
-        <v>531</v>
+        <v>482</v>
+      </c>
+      <c r="D472" t="s">
+        <v>128</v>
       </c>
       <c r="E472" t="s">
-        <v>497</v>
+        <v>481</v>
       </c>
       <c r="F472" t="s">
-        <v>527</v>
+        <v>64</v>
       </c>
     </row>
     <row r="473" spans="1:6" x14ac:dyDescent="0.35">
@@ -10977,16 +11014,16 @@
         <v>162</v>
       </c>
       <c r="B473" s="1" t="s">
-        <v>535</v>
+        <v>232</v>
       </c>
       <c r="D473" t="s">
-        <v>345</v>
+        <v>128</v>
       </c>
       <c r="E473" t="s">
-        <v>532</v>
+        <v>193</v>
       </c>
       <c r="F473" t="s">
-        <v>533</v>
+        <v>206</v>
       </c>
     </row>
     <row r="474" spans="1:6" x14ac:dyDescent="0.35">
@@ -10994,7 +11031,7 @@
         <v>162</v>
       </c>
       <c r="B474" s="1" t="s">
-        <v>528</v>
+        <v>502</v>
       </c>
       <c r="D474" t="s">
         <v>144</v>
@@ -11003,6 +11040,94 @@
         <v>497</v>
       </c>
       <c r="F474" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="475" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A475" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B475" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C475" t="s">
+        <v>415</v>
+      </c>
+      <c r="D475">
+        <v>1</v>
+      </c>
+      <c r="E475" t="s">
+        <v>532</v>
+      </c>
+      <c r="F475" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="476" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A476" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B476" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C476" t="s">
+        <v>506</v>
+      </c>
+      <c r="E476" t="s">
+        <v>497</v>
+      </c>
+      <c r="F476" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="477" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A477" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B477" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C477" t="s">
+        <v>531</v>
+      </c>
+      <c r="E477" t="s">
+        <v>497</v>
+      </c>
+      <c r="F477" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="478" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A478" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B478" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="D478" t="s">
+        <v>345</v>
+      </c>
+      <c r="E478" t="s">
+        <v>532</v>
+      </c>
+      <c r="F478" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="479" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A479" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B479" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="D479" t="s">
+        <v>144</v>
+      </c>
+      <c r="E479" t="s">
+        <v>497</v>
+      </c>
+      <c r="F479" t="s">
         <v>529</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[Word] (Selection) Add snippet for getNextRange and getPreviousRange (#1065)
* [Word] (Selection) Add snippet for getNextRange and getPreviousRange

* Update description
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/word.xlsx
+++ b/snippet-extractor-metadata/word.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14863876-029E-4319-A045-C665BA386D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23473AC-1060-41C5-AA4D-116ACC111178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2371" uniqueCount="613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2396" uniqueCount="623">
   <si>
     <t>Class</t>
   </si>
@@ -1859,6 +1859,36 @@
   </si>
   <si>
     <t>SelectionInsertFormulaOptions</t>
+  </si>
+  <si>
+    <t>getNextRange</t>
+  </si>
+  <si>
+    <t>getPreviousRange</t>
+  </si>
+  <si>
+    <t>word-selection-get-previous-next-range</t>
+  </si>
+  <si>
+    <t>SelectionNextOptions</t>
+  </si>
+  <si>
+    <t>SelectionPreviousOptions</t>
+  </si>
+  <si>
+    <t>getNextWord</t>
+  </si>
+  <si>
+    <t>getPreviousSentence</t>
+  </si>
+  <si>
+    <t>getPreviousWord</t>
+  </si>
+  <si>
+    <t>getNextParagraph</t>
+  </si>
+  <si>
+    <t>OperationUnit</t>
   </si>
 </sst>
 </file>
@@ -1907,7 +1937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1918,6 +1948,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1973,8 +2004,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F474" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:F474" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F479" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:F479" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{1DA12987-AB2C-4056-A643-B1229DC856C5}" name="Package" dataDxfId="4"/>
     <tableColumn id="1" xr3:uid="{0CD83AD1-F92A-407D-8460-4E881461FD01}" name="Class" dataDxfId="3"/>
@@ -2284,7 +2315,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F474"/>
+  <dimension ref="A1:F479"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="25.08984375" bestFit="1" customWidth="1"/>
@@ -6119,14 +6150,14 @@
       <c r="B210" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C210" s="5" t="s">
+      <c r="C210" s="2" t="s">
         <v>605</v>
       </c>
       <c r="D210" s="2"/>
-      <c r="E210" s="5" t="s">
+      <c r="E210" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="F210" s="5" t="s">
+      <c r="F210" s="2" t="s">
         <v>608</v>
       </c>
     </row>
@@ -7413,20 +7444,21 @@
       </c>
     </row>
     <row r="281" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A281" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B281" s="1" t="s">
-        <v>411</v>
-      </c>
+      <c r="A281" t="s">
+        <v>162</v>
+      </c>
+      <c r="B281" s="4" t="s">
+        <v>622</v>
+      </c>
+      <c r="C281" s="6"/>
       <c r="D281" t="s">
         <v>128</v>
       </c>
-      <c r="E281" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="F281" s="2" t="s">
-        <v>375</v>
+      <c r="E281" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F281" s="5" t="s">
+        <v>618</v>
       </c>
     </row>
     <row r="282" spans="1:6" x14ac:dyDescent="0.35">
@@ -7434,16 +7466,16 @@
         <v>162</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>499</v>
+        <v>411</v>
       </c>
       <c r="D282" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="E282" s="2" t="s">
-        <v>497</v>
+        <v>374</v>
       </c>
       <c r="F282" s="2" t="s">
-        <v>498</v>
+        <v>375</v>
       </c>
     </row>
     <row r="283" spans="1:6" x14ac:dyDescent="0.35">
@@ -7453,11 +7485,8 @@
       <c r="B283" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="C283" t="s">
-        <v>115</v>
-      </c>
-      <c r="D283">
-        <v>1</v>
+      <c r="D283" t="s">
+        <v>144</v>
       </c>
       <c r="E283" s="2" t="s">
         <v>497</v>
@@ -7474,13 +7503,16 @@
         <v>499</v>
       </c>
       <c r="C284" t="s">
-        <v>500</v>
+        <v>115</v>
+      </c>
+      <c r="D284">
+        <v>1</v>
       </c>
       <c r="E284" s="2" t="s">
         <v>497</v>
       </c>
       <c r="F284" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="285" spans="1:6" x14ac:dyDescent="0.35">
@@ -7488,16 +7520,16 @@
         <v>162</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="D285" t="s">
-        <v>144</v>
+        <v>499</v>
+      </c>
+      <c r="C285" t="s">
+        <v>500</v>
       </c>
       <c r="E285" s="2" t="s">
         <v>497</v>
       </c>
       <c r="F285" s="2" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
     </row>
     <row r="286" spans="1:6" x14ac:dyDescent="0.35">
@@ -7505,7 +7537,7 @@
         <v>162</v>
       </c>
       <c r="B286" s="1" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="D286" t="s">
         <v>144</v>
@@ -7514,7 +7546,7 @@
         <v>497</v>
       </c>
       <c r="F286" s="2" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
     </row>
     <row r="287" spans="1:6" x14ac:dyDescent="0.35">
@@ -7524,8 +7556,8 @@
       <c r="B287" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="C287" t="s">
-        <v>508</v>
+      <c r="D287" t="s">
+        <v>144</v>
       </c>
       <c r="E287" s="2" t="s">
         <v>497</v>
@@ -7542,13 +7574,13 @@
         <v>504</v>
       </c>
       <c r="C288" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E288" s="2" t="s">
         <v>497</v>
       </c>
       <c r="F288" s="2" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
     </row>
     <row r="289" spans="1:6" x14ac:dyDescent="0.35">
@@ -7556,34 +7588,33 @@
         <v>162</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="D289" t="s">
-        <v>144</v>
+        <v>504</v>
+      </c>
+      <c r="C289" t="s">
+        <v>509</v>
       </c>
       <c r="E289" s="2" t="s">
         <v>497</v>
       </c>
       <c r="F289" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A290" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="D290" t="s">
+        <v>144</v>
+      </c>
+      <c r="E290" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="F290" s="2" t="s">
         <v>527</v>
-      </c>
-    </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A290" t="s">
-        <v>162</v>
-      </c>
-      <c r="B290" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C290" s="2"/>
-      <c r="D290" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E290" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F290" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="291" spans="1:6" x14ac:dyDescent="0.35">
@@ -7593,77 +7624,75 @@
       <c r="B291" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C291" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D291" s="2">
-        <v>1</v>
+      <c r="C291" s="2"/>
+      <c r="D291" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E291" s="1" t="s">
         <v>79</v>
       </c>
       <c r="F291" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="292" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A292" s="1" t="s">
+      <c r="A292" t="s">
         <v>162</v>
       </c>
       <c r="B292" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>360</v>
+        <v>115</v>
       </c>
       <c r="D292" s="2">
         <v>1</v>
       </c>
       <c r="E292" s="1" t="s">
-        <v>350</v>
+        <v>79</v>
       </c>
       <c r="F292" s="2" t="s">
-        <v>360</v>
+        <v>12</v>
       </c>
     </row>
     <row r="293" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A293" t="s">
+      <c r="A293" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B293" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>29</v>
+        <v>360</v>
       </c>
       <c r="D293" s="2">
         <v>1</v>
       </c>
-      <c r="E293" s="2" t="s">
-        <v>75</v>
+      <c r="E293" s="1" t="s">
+        <v>350</v>
       </c>
       <c r="F293" s="2" t="s">
-        <v>28</v>
+        <v>360</v>
       </c>
     </row>
     <row r="294" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A294" s="1" t="s">
+      <c r="A294" t="s">
         <v>162</v>
       </c>
       <c r="B294" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D294" s="2">
         <v>1</v>
       </c>
       <c r="E294" s="2" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="F294" s="2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="295" spans="1:6" x14ac:dyDescent="0.35">
@@ -7674,36 +7703,36 @@
         <v>10</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>556</v>
+        <v>36</v>
       </c>
       <c r="D295" s="2">
         <v>1</v>
       </c>
       <c r="E295" s="2" t="s">
-        <v>570</v>
+        <v>43</v>
       </c>
       <c r="F295" s="2" t="s">
-        <v>151</v>
+        <v>42</v>
       </c>
     </row>
     <row r="296" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A296" t="s">
+      <c r="A296" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B296" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>13</v>
+        <v>556</v>
       </c>
       <c r="D296" s="2">
         <v>1</v>
       </c>
       <c r="E296" s="2" t="s">
-        <v>81</v>
+        <v>570</v>
       </c>
       <c r="F296" s="2" t="s">
-        <v>22</v>
+        <v>151</v>
       </c>
     </row>
     <row r="297" spans="1:6" x14ac:dyDescent="0.35">
@@ -7714,16 +7743,16 @@
         <v>10</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>512</v>
+        <v>13</v>
       </c>
       <c r="D297" s="2">
         <v>1</v>
       </c>
       <c r="E297" s="2" t="s">
-        <v>537</v>
+        <v>81</v>
       </c>
       <c r="F297" s="2" t="s">
-        <v>523</v>
+        <v>22</v>
       </c>
     </row>
     <row r="298" spans="1:6" x14ac:dyDescent="0.35">
@@ -7734,16 +7763,16 @@
         <v>10</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>48</v>
+        <v>512</v>
       </c>
       <c r="D298" s="2">
         <v>1</v>
       </c>
       <c r="E298" s="2" t="s">
-        <v>71</v>
+        <v>537</v>
       </c>
       <c r="F298" s="2" t="s">
-        <v>47</v>
+        <v>523</v>
       </c>
     </row>
     <row r="299" spans="1:6" x14ac:dyDescent="0.35">
@@ -7763,7 +7792,7 @@
         <v>71</v>
       </c>
       <c r="F299" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.35">
@@ -7773,17 +7802,17 @@
       <c r="B300" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C300" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D300" s="1">
+      <c r="C300" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D300" s="2">
         <v>1</v>
       </c>
       <c r="E300" s="2" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="F300" s="2" t="s">
-        <v>7</v>
+        <v>49</v>
       </c>
     </row>
     <row r="301" spans="1:6" x14ac:dyDescent="0.35">
@@ -7793,17 +7822,17 @@
       <c r="B301" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C301" s="2" t="s">
+      <c r="C301" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D301" s="2">
+      <c r="D301" s="1">
         <v>1</v>
       </c>
       <c r="E301" s="2" t="s">
         <v>83</v>
       </c>
       <c r="F301" s="2" t="s">
-        <v>66</v>
+        <v>7</v>
       </c>
     </row>
     <row r="302" spans="1:6" x14ac:dyDescent="0.35">
@@ -7814,16 +7843,16 @@
         <v>10</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="D302" s="2">
         <v>1</v>
       </c>
       <c r="E302" s="2" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F302" s="2" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
     </row>
     <row r="303" spans="1:6" x14ac:dyDescent="0.35">
@@ -7834,16 +7863,16 @@
         <v>10</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D303" s="2">
         <v>1</v>
       </c>
       <c r="E303" s="2" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="F303" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="304" spans="1:6" x14ac:dyDescent="0.35">
@@ -7854,14 +7883,16 @@
         <v>10</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D304" s="2"/>
+        <v>59</v>
+      </c>
+      <c r="D304" s="2">
+        <v>1</v>
+      </c>
       <c r="E304" s="2" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="F304" s="2" t="s">
-        <v>18</v>
+        <v>58</v>
       </c>
     </row>
     <row r="305" spans="1:6" x14ac:dyDescent="0.35">
@@ -7872,14 +7903,14 @@
         <v>10</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D305" s="2"/>
       <c r="E305" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F305" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="306" spans="1:6" x14ac:dyDescent="0.35">
@@ -7890,86 +7921,86 @@
         <v>10</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D306" s="2"/>
       <c r="E306" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F306" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="307" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A307" s="1" t="s">
+      <c r="A307" t="s">
         <v>162</v>
       </c>
       <c r="B307" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>379</v>
+        <v>20</v>
       </c>
       <c r="D307" s="2"/>
       <c r="E307" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F307" s="2" t="s">
-        <v>380</v>
+        <v>16</v>
       </c>
     </row>
     <row r="308" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A308" s="3" t="s">
+      <c r="A308" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B308" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D308" s="2"/>
       <c r="E308" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F308" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="309" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A309" t="s">
+      <c r="A309" s="3" t="s">
         <v>162</v>
       </c>
       <c r="B309" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>17</v>
+        <v>381</v>
       </c>
       <c r="D309" s="2"/>
       <c r="E309" s="2" t="s">
         <v>80</v>
       </c>
       <c r="F309" s="2" t="s">
-        <v>17</v>
+        <v>382</v>
       </c>
     </row>
     <row r="310" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A310" s="1" t="s">
+      <c r="A310" t="s">
         <v>162</v>
       </c>
       <c r="B310" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>280</v>
+        <v>17</v>
       </c>
       <c r="D310" s="2"/>
       <c r="E310" s="2" t="s">
-        <v>269</v>
+        <v>80</v>
       </c>
       <c r="F310" s="2" t="s">
-        <v>279</v>
+        <v>17</v>
       </c>
     </row>
     <row r="311" spans="1:6" x14ac:dyDescent="0.35">
@@ -7980,32 +8011,32 @@
         <v>10</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>238</v>
+        <v>280</v>
       </c>
       <c r="D311" s="2"/>
       <c r="E311" s="2" t="s">
-        <v>82</v>
+        <v>269</v>
       </c>
       <c r="F311" s="2" t="s">
-        <v>240</v>
+        <v>279</v>
       </c>
     </row>
     <row r="312" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A312" t="s">
+      <c r="A312" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B312" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>8</v>
+        <v>238</v>
       </c>
       <c r="D312" s="2"/>
-      <c r="E312" s="1" t="s">
-        <v>79</v>
+      <c r="E312" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="F312" s="2" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
     </row>
     <row r="313" spans="1:6" x14ac:dyDescent="0.35">
@@ -8016,14 +8047,14 @@
         <v>10</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>369</v>
+        <v>8</v>
       </c>
       <c r="D313" s="2"/>
       <c r="E313" s="1" t="s">
-        <v>350</v>
+        <v>79</v>
       </c>
       <c r="F313" s="2" t="s">
-        <v>123</v>
+        <v>11</v>
       </c>
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.35">
@@ -8041,25 +8072,25 @@
         <v>350</v>
       </c>
       <c r="F314" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="315" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A315" t="s">
+        <v>162</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C315" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="D315" s="2"/>
+      <c r="E315" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F315" s="2" t="s">
         <v>324</v>
-      </c>
-    </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A315" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B315" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="C315" s="2"/>
-      <c r="D315" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="E315" s="1" t="s">
-        <v>318</v>
-      </c>
-      <c r="F315" s="2" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.35">
@@ -8077,7 +8108,7 @@
         <v>318</v>
       </c>
       <c r="F316" s="2" t="s">
-        <v>319</v>
+        <v>267</v>
       </c>
     </row>
     <row r="317" spans="1:6" x14ac:dyDescent="0.35">
@@ -8085,17 +8116,17 @@
         <v>162</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C317" s="2"/>
       <c r="D317" s="2" t="s">
         <v>345</v>
       </c>
       <c r="E317" s="1" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="F317" s="2" t="s">
-        <v>267</v>
+        <v>319</v>
       </c>
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.35">
@@ -8113,65 +8144,63 @@
         <v>322</v>
       </c>
       <c r="F318" s="2" t="s">
-        <v>324</v>
+        <v>267</v>
       </c>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A319" t="s">
+      <c r="A319" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>190</v>
+        <v>329</v>
       </c>
       <c r="C319" s="2"/>
       <c r="D319" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E319" s="2" t="s">
-        <v>70</v>
+        <v>345</v>
+      </c>
+      <c r="E319" s="1" t="s">
+        <v>322</v>
       </c>
       <c r="F319" s="2" t="s">
-        <v>175</v>
+        <v>324</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A320" s="1" t="s">
+      <c r="A320" t="s">
         <v>162</v>
       </c>
       <c r="B320" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C320" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D320" s="2">
-        <v>1</v>
-      </c>
-      <c r="E320" s="1" t="s">
-        <v>350</v>
+      <c r="C320" s="2"/>
+      <c r="D320" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E320" s="2" t="s">
+        <v>70</v>
       </c>
       <c r="F320" s="2" t="s">
-        <v>353</v>
+        <v>175</v>
       </c>
     </row>
     <row r="321" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A321" t="s">
+      <c r="A321" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B321" s="1" t="s">
         <v>190</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>176</v>
+        <v>100</v>
       </c>
       <c r="D321" s="2">
         <v>1</v>
       </c>
-      <c r="E321" s="2" t="s">
-        <v>70</v>
+      <c r="E321" s="1" t="s">
+        <v>350</v>
       </c>
       <c r="F321" s="2" t="s">
-        <v>175</v>
+        <v>353</v>
       </c>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.35">
@@ -8182,14 +8211,16 @@
         <v>190</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D322" s="2"/>
+        <v>176</v>
+      </c>
+      <c r="D322" s="2">
+        <v>1</v>
+      </c>
       <c r="E322" s="2" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="F322" s="2" t="s">
-        <v>58</v>
+        <v>175</v>
       </c>
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.35">
@@ -8197,17 +8228,17 @@
         <v>162</v>
       </c>
       <c r="B323" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="C323" s="2"/>
-      <c r="D323" s="2" t="s">
-        <v>345</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="C323" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D323" s="2"/>
       <c r="E323" s="2" t="s">
-        <v>323</v>
+        <v>57</v>
       </c>
       <c r="F323" s="2" t="s">
-        <v>267</v>
+        <v>58</v>
       </c>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.35">
@@ -8225,25 +8256,25 @@
         <v>323</v>
       </c>
       <c r="F324" s="2" t="s">
-        <v>325</v>
+        <v>267</v>
       </c>
     </row>
     <row r="325" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A325" s="1" t="s">
+      <c r="A325" t="s">
         <v>162</v>
       </c>
       <c r="B325" s="1" t="s">
-        <v>281</v>
+        <v>346</v>
       </c>
       <c r="C325" s="2"/>
       <c r="D325" s="2" t="s">
-        <v>144</v>
+        <v>345</v>
       </c>
       <c r="E325" s="2" t="s">
-        <v>269</v>
+        <v>323</v>
       </c>
       <c r="F325" s="2" t="s">
-        <v>294</v>
+        <v>325</v>
       </c>
     </row>
     <row r="326" spans="1:6" x14ac:dyDescent="0.35">
@@ -8253,10 +8284,10 @@
       <c r="B326" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="C326" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D326" s="2"/>
+      <c r="C326" s="2"/>
+      <c r="D326" s="2" t="s">
+        <v>144</v>
+      </c>
       <c r="E326" s="2" t="s">
         <v>269</v>
       </c>
@@ -8272,7 +8303,7 @@
         <v>281</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D327" s="2"/>
       <c r="E327" s="2" t="s">
@@ -8287,17 +8318,17 @@
         <v>162</v>
       </c>
       <c r="B328" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C328" s="2"/>
-      <c r="D328" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>281</v>
+      </c>
+      <c r="C328" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D328" s="2"/>
       <c r="E328" s="2" t="s">
-        <v>145</v>
+        <v>269</v>
       </c>
       <c r="F328" s="2" t="s">
-        <v>445</v>
+        <v>294</v>
       </c>
     </row>
     <row r="329" spans="1:6" x14ac:dyDescent="0.35">
@@ -8307,17 +8338,15 @@
       <c r="B329" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C329" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D329" s="2">
-        <v>1</v>
+      <c r="C329" s="2"/>
+      <c r="D329" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E329" s="2" t="s">
-        <v>227</v>
+        <v>145</v>
       </c>
       <c r="F329" s="2" t="s">
-        <v>228</v>
+        <v>445</v>
       </c>
     </row>
     <row r="330" spans="1:6" x14ac:dyDescent="0.35">
@@ -8328,36 +8357,36 @@
         <v>5</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>492</v>
+        <v>229</v>
       </c>
       <c r="D330" s="2">
         <v>1</v>
       </c>
       <c r="E330" s="2" t="s">
-        <v>79</v>
+        <v>227</v>
       </c>
       <c r="F330" s="2" t="s">
-        <v>12</v>
+        <v>228</v>
       </c>
     </row>
     <row r="331" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A331" t="s">
+      <c r="A331" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B331" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C331" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D331" s="1">
+      <c r="C331" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="D331" s="2">
         <v>1</v>
       </c>
       <c r="E331" s="2" t="s">
-        <v>145</v>
+        <v>79</v>
       </c>
       <c r="F331" s="2" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
     </row>
     <row r="332" spans="1:6" x14ac:dyDescent="0.35">
@@ -8368,16 +8397,16 @@
         <v>5</v>
       </c>
       <c r="C332" s="1" t="s">
-        <v>395</v>
+        <v>107</v>
       </c>
       <c r="D332" s="1">
         <v>1</v>
       </c>
       <c r="E332" s="2" t="s">
-        <v>393</v>
+        <v>145</v>
       </c>
       <c r="F332" s="2" t="s">
-        <v>427</v>
+        <v>108</v>
       </c>
     </row>
     <row r="333" spans="1:6" x14ac:dyDescent="0.35">
@@ -8388,16 +8417,16 @@
         <v>5</v>
       </c>
       <c r="C333" s="1" t="s">
-        <v>115</v>
+        <v>395</v>
       </c>
       <c r="D333" s="1">
         <v>1</v>
       </c>
       <c r="E333" s="2" t="s">
-        <v>494</v>
+        <v>393</v>
       </c>
       <c r="F333" s="2" t="s">
-        <v>462</v>
+        <v>427</v>
       </c>
     </row>
     <row r="334" spans="1:6" x14ac:dyDescent="0.35">
@@ -8408,16 +8437,16 @@
         <v>5</v>
       </c>
       <c r="C334" s="1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D334" s="1">
         <v>1</v>
       </c>
       <c r="E334" s="2" t="s">
-        <v>147</v>
+        <v>494</v>
       </c>
       <c r="F334" s="2" t="s">
-        <v>121</v>
+        <v>462</v>
       </c>
     </row>
     <row r="335" spans="1:6" x14ac:dyDescent="0.35">
@@ -8428,16 +8457,16 @@
         <v>5</v>
       </c>
       <c r="C335" s="1" t="s">
-        <v>14</v>
+        <v>121</v>
       </c>
       <c r="D335" s="1">
         <v>1</v>
       </c>
-      <c r="E335" s="1" t="s">
-        <v>79</v>
+      <c r="E335" s="2" t="s">
+        <v>147</v>
       </c>
       <c r="F335" s="2" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
     </row>
     <row r="336" spans="1:6" x14ac:dyDescent="0.35">
@@ -8448,16 +8477,16 @@
         <v>5</v>
       </c>
       <c r="C336" s="1" t="s">
-        <v>106</v>
+        <v>14</v>
       </c>
       <c r="D336" s="1">
         <v>1</v>
       </c>
       <c r="E336" s="1" t="s">
-        <v>145</v>
+        <v>79</v>
       </c>
       <c r="F336" s="2" t="s">
-        <v>106</v>
+        <v>12</v>
       </c>
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.35">
@@ -8468,56 +8497,56 @@
         <v>5</v>
       </c>
       <c r="C337" s="1" t="s">
-        <v>36</v>
+        <v>106</v>
       </c>
       <c r="D337" s="1">
         <v>1</v>
       </c>
-      <c r="E337" s="2" t="s">
-        <v>82</v>
+      <c r="E337" s="1" t="s">
+        <v>145</v>
       </c>
       <c r="F337" s="2" t="s">
-        <v>35</v>
+        <v>106</v>
       </c>
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A338" s="1" t="s">
+      <c r="A338" t="s">
         <v>162</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C338" s="1" t="s">
-        <v>283</v>
+        <v>36</v>
       </c>
       <c r="D338" s="1">
         <v>1</v>
       </c>
       <c r="E338" s="2" t="s">
-        <v>163</v>
+        <v>82</v>
       </c>
       <c r="F338" s="2" t="s">
-        <v>284</v>
+        <v>35</v>
       </c>
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A339" t="s">
+      <c r="A339" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C339" s="1" t="s">
-        <v>88</v>
+        <v>283</v>
       </c>
       <c r="D339" s="1">
         <v>1</v>
       </c>
-      <c r="E339" s="1" t="s">
-        <v>146</v>
+      <c r="E339" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="F339" s="2" t="s">
-        <v>88</v>
+        <v>284</v>
       </c>
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.35">
@@ -8528,16 +8557,16 @@
         <v>5</v>
       </c>
       <c r="C340" s="1" t="s">
-        <v>313</v>
+        <v>88</v>
       </c>
       <c r="D340" s="1">
         <v>1</v>
       </c>
       <c r="E340" s="1" t="s">
-        <v>537</v>
+        <v>146</v>
       </c>
       <c r="F340" s="2" t="s">
-        <v>521</v>
+        <v>88</v>
       </c>
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.35">
@@ -8557,7 +8586,7 @@
         <v>537</v>
       </c>
       <c r="F341" s="2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.35">
@@ -8568,16 +8597,16 @@
         <v>5</v>
       </c>
       <c r="C342" s="1" t="s">
-        <v>556</v>
+        <v>313</v>
       </c>
       <c r="D342" s="1">
         <v>1</v>
       </c>
       <c r="E342" s="1" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F342" s="2" t="s">
-        <v>561</v>
+        <v>524</v>
       </c>
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.35">
@@ -8588,16 +8617,16 @@
         <v>5</v>
       </c>
       <c r="C343" s="1" t="s">
-        <v>512</v>
+        <v>556</v>
       </c>
       <c r="D343" s="1">
         <v>1</v>
       </c>
       <c r="E343" s="1" t="s">
-        <v>537</v>
+        <v>555</v>
       </c>
       <c r="F343" s="2" t="s">
-        <v>511</v>
+        <v>561</v>
       </c>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.35">
@@ -8608,31 +8637,34 @@
         <v>5</v>
       </c>
       <c r="C344" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D344" s="1"/>
+        <v>512</v>
+      </c>
+      <c r="D344" s="1">
+        <v>1</v>
+      </c>
       <c r="E344" s="1" t="s">
-        <v>146</v>
+        <v>537</v>
       </c>
       <c r="F344" s="2" t="s">
-        <v>96</v>
+        <v>511</v>
       </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A345" s="1" t="s">
+      <c r="A345" t="s">
         <v>162</v>
       </c>
       <c r="B345" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C345" t="s">
-        <v>428</v>
-      </c>
-      <c r="E345" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="F345" t="s">
-        <v>422</v>
+      <c r="C345" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D345" s="1"/>
+      <c r="E345" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F345" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.35">
@@ -8642,15 +8674,14 @@
       <c r="B346" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C346" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D346" s="2"/>
+      <c r="C346" t="s">
+        <v>428</v>
+      </c>
       <c r="E346" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F346" s="2" t="s">
-        <v>239</v>
+        <v>393</v>
+      </c>
+      <c r="F346" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="347" spans="1:6" x14ac:dyDescent="0.35">
@@ -8658,53 +8689,53 @@
         <v>162</v>
       </c>
       <c r="B347" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C347" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D347" s="2"/>
+      <c r="E347" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F347" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="348" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A348" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B348" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="C347" s="2"/>
-      <c r="D347" s="2" t="s">
+      <c r="C348" s="2"/>
+      <c r="D348" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E347" s="2" t="s">
+      <c r="E348" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F347" s="2" t="s">
+      <c r="F348" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="348" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A348" t="s">
-        <v>162</v>
-      </c>
-      <c r="B348" s="1" t="s">
+    <row r="349" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A349" t="s">
+        <v>162</v>
+      </c>
+      <c r="B349" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="C348" s="1"/>
-      <c r="D348" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E348" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F348" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="349" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A349" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B349" s="1" t="s">
-        <v>575</v>
       </c>
       <c r="C349" s="1"/>
       <c r="D349" s="1" t="s">
         <v>128</v>
       </c>
       <c r="E349" s="1" t="s">
-        <v>570</v>
+        <v>79</v>
       </c>
       <c r="F349" s="2" t="s">
-        <v>576</v>
+        <v>12</v>
       </c>
     </row>
     <row r="350" spans="1:6" x14ac:dyDescent="0.35">
@@ -8712,7 +8743,7 @@
         <v>162</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C350" s="1"/>
       <c r="D350" s="1" t="s">
@@ -8722,7 +8753,7 @@
         <v>570</v>
       </c>
       <c r="F350" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="351" spans="1:6" x14ac:dyDescent="0.35">
@@ -8730,7 +8761,7 @@
         <v>162</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C351" s="1"/>
       <c r="D351" s="1" t="s">
@@ -8740,7 +8771,7 @@
         <v>570</v>
       </c>
       <c r="F351" s="2" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="352" spans="1:6" x14ac:dyDescent="0.35">
@@ -8748,17 +8779,17 @@
         <v>162</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>418</v>
+        <v>579</v>
       </c>
       <c r="C352" s="1"/>
       <c r="D352" s="1" t="s">
         <v>128</v>
       </c>
       <c r="E352" s="1" t="s">
-        <v>413</v>
+        <v>570</v>
       </c>
       <c r="F352" s="2" t="s">
-        <v>414</v>
+        <v>576</v>
       </c>
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.35">
@@ -8766,37 +8797,35 @@
         <v>162</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>534</v>
+        <v>418</v>
       </c>
       <c r="C353" s="1"/>
       <c r="D353" s="1" t="s">
         <v>128</v>
       </c>
       <c r="E353" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F353" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="354" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A354" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C354" s="1"/>
+      <c r="D354" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E354" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="F353" s="2" t="s">
+      <c r="F354" s="2" t="s">
         <v>533</v>
-      </c>
-    </row>
-    <row r="354" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A354" t="s">
-        <v>162</v>
-      </c>
-      <c r="B354" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C354" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D354" s="2">
-        <v>2</v>
-      </c>
-      <c r="E354" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F354" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="355" spans="1:6" x14ac:dyDescent="0.35">
@@ -8806,17 +8835,17 @@
       <c r="B355" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C355" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D355" s="1">
-        <v>1</v>
+      <c r="C355" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D355" s="2">
+        <v>2</v>
       </c>
       <c r="E355" s="2" t="s">
         <v>78</v>
       </c>
       <c r="F355" s="2" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.35">
@@ -8826,15 +8855,17 @@
       <c r="B356" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C356" s="1"/>
-      <c r="D356" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="E356" s="1" t="s">
-        <v>140</v>
+      <c r="C356" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D356" s="1">
+        <v>1</v>
+      </c>
+      <c r="E356" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="F356" s="2" t="s">
-        <v>141</v>
+        <v>69</v>
       </c>
     </row>
     <row r="357" spans="1:6" x14ac:dyDescent="0.35">
@@ -8842,73 +8873,73 @@
         <v>162</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C357" s="2"/>
-      <c r="D357" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C357" s="1"/>
+      <c r="D357" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E357" s="2" t="s">
+      <c r="E357" s="1" t="s">
         <v>140</v>
       </c>
       <c r="F357" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="358" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
         <v>162</v>
       </c>
-      <c r="B358" s="4" t="s">
-        <v>609</v>
-      </c>
-      <c r="C358" s="5"/>
+      <c r="B358" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C358" s="2"/>
       <c r="D358" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E358" s="5" t="s">
-        <v>606</v>
-      </c>
-      <c r="F358" s="5" t="s">
-        <v>608</v>
+      <c r="E358" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F358" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="359" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
         <v>162</v>
       </c>
-      <c r="B359" s="4" t="s">
+      <c r="B359" s="1" t="s">
         <v>609</v>
       </c>
-      <c r="C359" s="5" t="s">
-        <v>610</v>
-      </c>
-      <c r="D359" s="2">
-        <v>1</v>
-      </c>
-      <c r="E359" s="5" t="s">
+      <c r="C359" s="2"/>
+      <c r="D359" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E359" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="F359" s="5" t="s">
-        <v>607</v>
+      <c r="F359" s="2" t="s">
+        <v>608</v>
       </c>
     </row>
     <row r="360" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
         <v>162</v>
       </c>
-      <c r="B360" s="4" t="s">
-        <v>612</v>
-      </c>
-      <c r="C360" s="5"/>
-      <c r="D360" s="2" t="s">
-        <v>345</v>
+      <c r="B360" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="C360" s="5" t="s">
+        <v>613</v>
+      </c>
+      <c r="D360" s="2">
+        <v>1</v>
       </c>
       <c r="E360" s="5" t="s">
-        <v>606</v>
+        <v>615</v>
       </c>
       <c r="F360" s="5" t="s">
-        <v>611</v>
+        <v>621</v>
       </c>
     </row>
     <row r="361" spans="1:6" x14ac:dyDescent="0.35">
@@ -8916,109 +8947,111 @@
         <v>162</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C361" s="2"/>
-      <c r="D361" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E361" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F361" s="2" t="s">
-        <v>49</v>
+        <v>609</v>
+      </c>
+      <c r="C361" s="5" t="s">
+        <v>614</v>
+      </c>
+      <c r="D361" s="2">
+        <v>1</v>
+      </c>
+      <c r="E361" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F361" s="5" t="s">
+        <v>619</v>
       </c>
     </row>
     <row r="362" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A362" s="1" t="s">
+      <c r="A362" t="s">
         <v>162</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="C362" s="2"/>
-      <c r="D362" s="2" t="s">
-        <v>144</v>
+        <v>609</v>
+      </c>
+      <c r="C362" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="D362" s="2">
+        <v>1</v>
       </c>
       <c r="E362" s="2" t="s">
-        <v>164</v>
+        <v>606</v>
       </c>
       <c r="F362" s="2" t="s">
-        <v>168</v>
+        <v>607</v>
       </c>
     </row>
     <row r="363" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A363" s="1" t="s">
+      <c r="A363" t="s">
         <v>162</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="C363" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="D363" s="2"/>
+        <v>612</v>
+      </c>
+      <c r="C363" s="2"/>
+      <c r="D363" s="2" t="s">
+        <v>345</v>
+      </c>
       <c r="E363" s="2" t="s">
-        <v>164</v>
+        <v>606</v>
       </c>
       <c r="F363" s="2" t="s">
-        <v>168</v>
+        <v>611</v>
       </c>
     </row>
     <row r="364" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B364" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="C364" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="D364" s="2"/>
-      <c r="E364" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="F364" s="2" t="s">
-        <v>168</v>
+      <c r="B364" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="C364" s="5"/>
+      <c r="D364" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="E364" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F364" s="5" t="s">
+        <v>618</v>
       </c>
     </row>
     <row r="365" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B365" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C365" s="2"/>
+      <c r="B365" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="C365" s="5"/>
       <c r="D365" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="E365" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="F365" s="2" t="s">
-        <v>166</v>
+        <v>345</v>
+      </c>
+      <c r="E365" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F365" s="5" t="s">
+        <v>620</v>
       </c>
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A366" s="1" t="s">
+      <c r="A366" t="s">
         <v>162</v>
       </c>
       <c r="B366" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C366" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D366" s="2">
-        <v>1</v>
+        <v>159</v>
+      </c>
+      <c r="C366" s="2"/>
+      <c r="D366" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="E366" s="2" t="s">
-        <v>164</v>
+        <v>71</v>
       </c>
       <c r="F366" s="2" t="s">
-        <v>168</v>
+        <v>49</v>
       </c>
     </row>
     <row r="367" spans="1:6" x14ac:dyDescent="0.35">
@@ -9026,17 +9059,17 @@
         <v>162</v>
       </c>
       <c r="B367" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C367" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D367" s="2"/>
+        <v>296</v>
+      </c>
+      <c r="C367" s="2"/>
+      <c r="D367" s="2" t="s">
+        <v>144</v>
+      </c>
       <c r="E367" s="2" t="s">
         <v>164</v>
       </c>
       <c r="F367" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="368" spans="1:6" x14ac:dyDescent="0.35">
@@ -9044,17 +9077,17 @@
         <v>162</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="C368" s="2"/>
-      <c r="D368" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>296</v>
+      </c>
+      <c r="C368" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D368" s="2"/>
       <c r="E368" s="2" t="s">
-        <v>269</v>
+        <v>164</v>
       </c>
       <c r="F368" s="2" t="s">
-        <v>489</v>
+        <v>168</v>
       </c>
     </row>
     <row r="369" spans="1:6" x14ac:dyDescent="0.35">
@@ -9062,17 +9095,17 @@
         <v>162</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="C369" s="2"/>
-      <c r="D369" s="2" t="s">
-        <v>128</v>
-      </c>
+        <v>296</v>
+      </c>
+      <c r="C369" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D369" s="2"/>
       <c r="E369" s="2" t="s">
-        <v>269</v>
+        <v>164</v>
       </c>
       <c r="F369" s="2" t="s">
-        <v>489</v>
+        <v>168</v>
       </c>
     </row>
     <row r="370" spans="1:6" x14ac:dyDescent="0.35">
@@ -9080,17 +9113,17 @@
         <v>162</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>516</v>
+        <v>167</v>
       </c>
       <c r="C370" s="2"/>
       <c r="D370" s="2" t="s">
         <v>144</v>
       </c>
       <c r="E370" s="2" t="s">
-        <v>537</v>
+        <v>164</v>
       </c>
       <c r="F370" s="2" t="s">
-        <v>519</v>
+        <v>166</v>
       </c>
     </row>
     <row r="371" spans="1:6" x14ac:dyDescent="0.35">
@@ -9098,19 +9131,19 @@
         <v>162</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>516</v>
+        <v>167</v>
       </c>
       <c r="C371" s="2" t="s">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="D371" s="2">
         <v>1</v>
       </c>
       <c r="E371" s="2" t="s">
-        <v>537</v>
+        <v>164</v>
       </c>
       <c r="F371" s="2" t="s">
-        <v>522</v>
+        <v>168</v>
       </c>
     </row>
     <row r="372" spans="1:6" x14ac:dyDescent="0.35">
@@ -9118,19 +9151,17 @@
         <v>162</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>516</v>
+        <v>167</v>
       </c>
       <c r="C372" s="2" t="s">
-        <v>583</v>
-      </c>
-      <c r="D372" s="2">
-        <v>1</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="D372" s="2"/>
       <c r="E372" s="2" t="s">
-        <v>570</v>
+        <v>164</v>
       </c>
       <c r="F372" s="2" t="s">
-        <v>584</v>
+        <v>169</v>
       </c>
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.35">
@@ -9138,19 +9169,17 @@
         <v>162</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="C373" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="D373" s="2">
-        <v>1</v>
+        <v>491</v>
+      </c>
+      <c r="C373" s="2"/>
+      <c r="D373" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E373" s="2" t="s">
-        <v>570</v>
+        <v>269</v>
       </c>
       <c r="F373" s="2" t="s">
-        <v>584</v>
+        <v>489</v>
       </c>
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.35">
@@ -9158,19 +9187,17 @@
         <v>162</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="C374" s="2" t="s">
-        <v>587</v>
-      </c>
-      <c r="D374" s="2">
-        <v>1</v>
+        <v>490</v>
+      </c>
+      <c r="C374" s="2"/>
+      <c r="D374" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="E374" s="2" t="s">
-        <v>570</v>
+        <v>269</v>
       </c>
       <c r="F374" s="2" t="s">
-        <v>581</v>
+        <v>489</v>
       </c>
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.35">
@@ -9180,17 +9207,15 @@
       <c r="B375" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="C375" s="2" t="s">
-        <v>588</v>
-      </c>
-      <c r="D375" s="2">
-        <v>1</v>
+      <c r="C375" s="2"/>
+      <c r="D375" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E375" s="2" t="s">
-        <v>570</v>
+        <v>537</v>
       </c>
       <c r="F375" s="2" t="s">
-        <v>581</v>
+        <v>519</v>
       </c>
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.35">
@@ -9201,16 +9226,16 @@
         <v>516</v>
       </c>
       <c r="C376" s="2" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
       <c r="D376" s="2">
         <v>1</v>
       </c>
       <c r="E376" s="2" t="s">
-        <v>570</v>
+        <v>537</v>
       </c>
       <c r="F376" s="2" t="s">
-        <v>571</v>
+        <v>522</v>
       </c>
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.35">
@@ -9221,14 +9246,16 @@
         <v>516</v>
       </c>
       <c r="C377" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="D377" s="2"/>
+        <v>583</v>
+      </c>
+      <c r="D377" s="2">
+        <v>1</v>
+      </c>
       <c r="E377" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F377" s="2" t="s">
-        <v>520</v>
+        <v>584</v>
       </c>
     </row>
     <row r="378" spans="1:6" x14ac:dyDescent="0.35">
@@ -9239,14 +9266,16 @@
         <v>516</v>
       </c>
       <c r="C378" s="2" t="s">
-        <v>597</v>
-      </c>
-      <c r="D378" s="2"/>
+        <v>585</v>
+      </c>
+      <c r="D378" s="2">
+        <v>1</v>
+      </c>
       <c r="E378" s="2" t="s">
-        <v>595</v>
+        <v>570</v>
       </c>
       <c r="F378" s="2" t="s">
-        <v>596</v>
+        <v>584</v>
       </c>
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.35">
@@ -9257,14 +9286,16 @@
         <v>516</v>
       </c>
       <c r="C379" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="D379" s="2"/>
+        <v>587</v>
+      </c>
+      <c r="D379" s="2">
+        <v>1</v>
+      </c>
       <c r="E379" s="2" t="s">
-        <v>555</v>
+        <v>570</v>
       </c>
       <c r="F379" s="2" t="s">
-        <v>564</v>
+        <v>581</v>
       </c>
     </row>
     <row r="380" spans="1:6" x14ac:dyDescent="0.35">
@@ -9275,14 +9306,16 @@
         <v>516</v>
       </c>
       <c r="C380" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="D380" s="2"/>
+        <v>588</v>
+      </c>
+      <c r="D380" s="2">
+        <v>1</v>
+      </c>
       <c r="E380" s="2" t="s">
-        <v>555</v>
+        <v>570</v>
       </c>
       <c r="F380" s="2" t="s">
-        <v>559</v>
+        <v>581</v>
       </c>
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.35">
@@ -9293,14 +9326,16 @@
         <v>516</v>
       </c>
       <c r="C381" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="D381" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="D381" s="2">
+        <v>1</v>
+      </c>
       <c r="E381" s="2" t="s">
         <v>570</v>
       </c>
       <c r="F381" s="2" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
     </row>
     <row r="382" spans="1:6" x14ac:dyDescent="0.35">
@@ -9311,14 +9346,14 @@
         <v>516</v>
       </c>
       <c r="C382" s="2" t="s">
-        <v>589</v>
+        <v>104</v>
       </c>
       <c r="D382" s="2"/>
       <c r="E382" s="2" t="s">
-        <v>570</v>
+        <v>537</v>
       </c>
       <c r="F382" s="2" t="s">
-        <v>576</v>
+        <v>520</v>
       </c>
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.35">
@@ -9329,14 +9364,14 @@
         <v>516</v>
       </c>
       <c r="C383" s="2" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="D383" s="2"/>
       <c r="E383" s="2" t="s">
-        <v>570</v>
+        <v>595</v>
       </c>
       <c r="F383" s="2" t="s">
-        <v>578</v>
+        <v>596</v>
       </c>
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.35">
@@ -9347,14 +9382,14 @@
         <v>516</v>
       </c>
       <c r="C384" s="2" t="s">
-        <v>590</v>
+        <v>563</v>
       </c>
       <c r="D384" s="2"/>
       <c r="E384" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F384" s="2" t="s">
-        <v>576</v>
+        <v>564</v>
       </c>
     </row>
     <row r="385" spans="1:6" x14ac:dyDescent="0.35">
@@ -9365,14 +9400,14 @@
         <v>516</v>
       </c>
       <c r="C385" s="2" t="s">
-        <v>592</v>
+        <v>558</v>
       </c>
       <c r="D385" s="2"/>
       <c r="E385" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F385" s="2" t="s">
-        <v>578</v>
+        <v>559</v>
       </c>
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.35">
@@ -9383,14 +9418,14 @@
         <v>516</v>
       </c>
       <c r="C386" s="2" t="s">
-        <v>586</v>
+        <v>593</v>
       </c>
       <c r="D386" s="2"/>
       <c r="E386" s="2" t="s">
         <v>570</v>
       </c>
       <c r="F386" s="2" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
     </row>
     <row r="387" spans="1:6" x14ac:dyDescent="0.35">
@@ -9401,14 +9436,14 @@
         <v>516</v>
       </c>
       <c r="C387" s="2" t="s">
-        <v>538</v>
+        <v>589</v>
       </c>
       <c r="D387" s="2"/>
       <c r="E387" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F387" s="2" t="s">
-        <v>539</v>
+        <v>576</v>
       </c>
     </row>
     <row r="388" spans="1:6" x14ac:dyDescent="0.35">
@@ -9419,14 +9454,14 @@
         <v>516</v>
       </c>
       <c r="C388" s="2" t="s">
-        <v>541</v>
+        <v>591</v>
       </c>
       <c r="D388" s="2"/>
       <c r="E388" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F388" s="2" t="s">
-        <v>542</v>
+        <v>578</v>
       </c>
     </row>
     <row r="389" spans="1:6" x14ac:dyDescent="0.35">
@@ -9437,14 +9472,14 @@
         <v>516</v>
       </c>
       <c r="C389" s="2" t="s">
-        <v>94</v>
+        <v>590</v>
       </c>
       <c r="D389" s="2"/>
       <c r="E389" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F389" s="2" t="s">
-        <v>514</v>
+        <v>576</v>
       </c>
     </row>
     <row r="390" spans="1:6" x14ac:dyDescent="0.35">
@@ -9452,17 +9487,17 @@
         <v>162</v>
       </c>
       <c r="B390" s="1" t="s">
-        <v>548</v>
-      </c>
-      <c r="C390" s="2"/>
-      <c r="D390" s="2" t="s">
-        <v>128</v>
-      </c>
+        <v>516</v>
+      </c>
+      <c r="C390" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="D390" s="2"/>
       <c r="E390" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F390" s="2" t="s">
-        <v>549</v>
+        <v>578</v>
       </c>
     </row>
     <row r="391" spans="1:6" x14ac:dyDescent="0.35">
@@ -9470,17 +9505,17 @@
         <v>162</v>
       </c>
       <c r="B391" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="C391" s="2"/>
-      <c r="D391" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>516</v>
+      </c>
+      <c r="C391" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="D391" s="2"/>
       <c r="E391" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F391" s="2" t="s">
-        <v>514</v>
+        <v>571</v>
       </c>
     </row>
     <row r="392" spans="1:6" x14ac:dyDescent="0.35">
@@ -9488,19 +9523,17 @@
         <v>162</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C392" s="2" t="s">
-        <v>554</v>
-      </c>
-      <c r="D392" s="2">
-        <v>1</v>
-      </c>
+        <v>538</v>
+      </c>
+      <c r="D392" s="2"/>
       <c r="E392" s="2" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F392" s="2" t="s">
-        <v>562</v>
+        <v>539</v>
       </c>
     </row>
     <row r="393" spans="1:6" x14ac:dyDescent="0.35">
@@ -9508,19 +9541,17 @@
         <v>162</v>
       </c>
       <c r="B393" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C393" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="D393" s="2">
-        <v>1</v>
-      </c>
+        <v>541</v>
+      </c>
+      <c r="D393" s="2"/>
       <c r="E393" s="2" t="s">
         <v>537</v>
       </c>
       <c r="F393" s="2" t="s">
-        <v>519</v>
+        <v>542</v>
       </c>
     </row>
     <row r="394" spans="1:6" x14ac:dyDescent="0.35">
@@ -9528,19 +9559,17 @@
         <v>162</v>
       </c>
       <c r="B394" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C394" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D394" s="2">
-        <v>1</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D394" s="2"/>
       <c r="E394" s="2" t="s">
         <v>537</v>
       </c>
       <c r="F394" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
     </row>
     <row r="395" spans="1:6" x14ac:dyDescent="0.35">
@@ -9548,19 +9577,17 @@
         <v>162</v>
       </c>
       <c r="B395" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="C395" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D395" s="2">
-        <v>1</v>
+        <v>548</v>
+      </c>
+      <c r="C395" s="2"/>
+      <c r="D395" s="2" t="s">
+        <v>128</v>
       </c>
       <c r="E395" s="2" t="s">
         <v>537</v>
       </c>
       <c r="F395" s="2" t="s">
-        <v>536</v>
+        <v>549</v>
       </c>
     </row>
     <row r="396" spans="1:6" x14ac:dyDescent="0.35">
@@ -9570,17 +9597,15 @@
       <c r="B396" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="C396" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="D396" s="2">
-        <v>1</v>
+      <c r="C396" s="2"/>
+      <c r="D396" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E396" s="2" t="s">
-        <v>570</v>
+        <v>537</v>
       </c>
       <c r="F396" s="2" t="s">
-        <v>571</v>
+        <v>514</v>
       </c>
     </row>
     <row r="397" spans="1:6" x14ac:dyDescent="0.35">
@@ -9588,17 +9613,19 @@
         <v>162</v>
       </c>
       <c r="B397" s="1" t="s">
-        <v>565</v>
-      </c>
-      <c r="C397" s="2"/>
-      <c r="D397" s="2" t="s">
-        <v>144</v>
+        <v>513</v>
+      </c>
+      <c r="C397" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="D397" s="2">
+        <v>1</v>
       </c>
       <c r="E397" s="2" t="s">
         <v>555</v>
       </c>
       <c r="F397" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="398" spans="1:6" x14ac:dyDescent="0.35">
@@ -9606,19 +9633,19 @@
         <v>162</v>
       </c>
       <c r="B398" s="1" t="s">
-        <v>565</v>
+        <v>513</v>
       </c>
       <c r="C398" s="2" t="s">
-        <v>301</v>
+        <v>518</v>
       </c>
       <c r="D398" s="2">
         <v>1</v>
       </c>
       <c r="E398" s="2" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F398" s="2" t="s">
-        <v>567</v>
+        <v>519</v>
       </c>
     </row>
     <row r="399" spans="1:6" x14ac:dyDescent="0.35">
@@ -9626,19 +9653,19 @@
         <v>162</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>565</v>
+        <v>513</v>
       </c>
       <c r="C399" s="2" t="s">
-        <v>568</v>
+        <v>100</v>
       </c>
       <c r="D399" s="2">
         <v>1</v>
       </c>
       <c r="E399" s="2" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F399" s="2" t="s">
-        <v>567</v>
+        <v>520</v>
       </c>
     </row>
     <row r="400" spans="1:6" x14ac:dyDescent="0.35">
@@ -9646,17 +9673,19 @@
         <v>162</v>
       </c>
       <c r="B400" s="1" t="s">
-        <v>566</v>
-      </c>
-      <c r="C400" s="2"/>
-      <c r="D400" s="2" t="s">
-        <v>128</v>
+        <v>513</v>
+      </c>
+      <c r="C400" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D400" s="2">
+        <v>1</v>
       </c>
       <c r="E400" s="2" t="s">
-        <v>555</v>
+        <v>537</v>
       </c>
       <c r="F400" s="2" t="s">
-        <v>564</v>
+        <v>536</v>
       </c>
     </row>
     <row r="401" spans="1:6" x14ac:dyDescent="0.35">
@@ -9664,11 +9693,13 @@
         <v>162</v>
       </c>
       <c r="B401" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="C401" s="2"/>
-      <c r="D401" s="2" t="s">
-        <v>144</v>
+        <v>513</v>
+      </c>
+      <c r="C401" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="D401" s="2">
+        <v>1</v>
       </c>
       <c r="E401" s="2" t="s">
         <v>570</v>
@@ -9682,19 +9713,17 @@
         <v>162</v>
       </c>
       <c r="B402" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="C402" s="2" t="s">
-        <v>573</v>
-      </c>
-      <c r="D402" s="2">
-        <v>1</v>
+        <v>565</v>
+      </c>
+      <c r="C402" s="2"/>
+      <c r="D402" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E402" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F402" s="2" t="s">
-        <v>574</v>
+        <v>564</v>
       </c>
     </row>
     <row r="403" spans="1:6" x14ac:dyDescent="0.35">
@@ -9702,17 +9731,19 @@
         <v>162</v>
       </c>
       <c r="B403" s="1" t="s">
-        <v>572</v>
+        <v>565</v>
       </c>
       <c r="C403" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="D403" s="2"/>
+        <v>301</v>
+      </c>
+      <c r="D403" s="2">
+        <v>1</v>
+      </c>
       <c r="E403" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F403" s="2" t="s">
-        <v>584</v>
+        <v>567</v>
       </c>
     </row>
     <row r="404" spans="1:6" x14ac:dyDescent="0.35">
@@ -9720,17 +9751,19 @@
         <v>162</v>
       </c>
       <c r="B404" s="1" t="s">
-        <v>580</v>
-      </c>
-      <c r="C404" s="2"/>
-      <c r="D404" s="2" t="s">
-        <v>128</v>
+        <v>565</v>
+      </c>
+      <c r="C404" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="D404" s="2">
+        <v>1</v>
       </c>
       <c r="E404" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F404" s="2" t="s">
-        <v>581</v>
+        <v>567</v>
       </c>
     </row>
     <row r="405" spans="1:6" x14ac:dyDescent="0.35">
@@ -9738,17 +9771,17 @@
         <v>162</v>
       </c>
       <c r="B405" s="1" t="s">
-        <v>582</v>
+        <v>566</v>
       </c>
       <c r="C405" s="2"/>
       <c r="D405" s="2" t="s">
         <v>128</v>
       </c>
       <c r="E405" s="2" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="F405" s="2" t="s">
-        <v>581</v>
+        <v>564</v>
       </c>
     </row>
     <row r="406" spans="1:6" x14ac:dyDescent="0.35">
@@ -9756,17 +9789,17 @@
         <v>162</v>
       </c>
       <c r="B406" s="1" t="s">
-        <v>550</v>
+        <v>572</v>
       </c>
       <c r="C406" s="2"/>
       <c r="D406" s="2" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E406" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F406" s="2" t="s">
-        <v>549</v>
+        <v>571</v>
       </c>
     </row>
     <row r="407" spans="1:6" x14ac:dyDescent="0.35">
@@ -9774,17 +9807,19 @@
         <v>162</v>
       </c>
       <c r="B407" s="1" t="s">
-        <v>551</v>
-      </c>
-      <c r="C407" s="2"/>
-      <c r="D407" s="2" t="s">
-        <v>128</v>
+        <v>572</v>
+      </c>
+      <c r="C407" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="D407" s="2">
+        <v>1</v>
       </c>
       <c r="E407" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F407" s="2" t="s">
-        <v>549</v>
+        <v>574</v>
       </c>
     </row>
     <row r="408" spans="1:6" x14ac:dyDescent="0.35">
@@ -9792,17 +9827,17 @@
         <v>162</v>
       </c>
       <c r="B408" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="C408" s="2"/>
-      <c r="D408" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>572</v>
+      </c>
+      <c r="C408" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D408" s="2"/>
       <c r="E408" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F408" s="2" t="s">
-        <v>542</v>
+        <v>584</v>
       </c>
     </row>
     <row r="409" spans="1:6" x14ac:dyDescent="0.35">
@@ -9810,17 +9845,17 @@
         <v>162</v>
       </c>
       <c r="B409" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="C409" s="2" t="s">
-        <v>544</v>
-      </c>
-      <c r="D409" s="2"/>
+        <v>580</v>
+      </c>
+      <c r="C409" s="2"/>
+      <c r="D409" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E409" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F409" s="2" t="s">
-        <v>547</v>
+        <v>581</v>
       </c>
     </row>
     <row r="410" spans="1:6" x14ac:dyDescent="0.35">
@@ -9828,17 +9863,17 @@
         <v>162</v>
       </c>
       <c r="B410" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="C410" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D410" s="2"/>
+        <v>582</v>
+      </c>
+      <c r="C410" s="2"/>
+      <c r="D410" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E410" s="2" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="F410" s="2" t="s">
-        <v>547</v>
+        <v>581</v>
       </c>
     </row>
     <row r="411" spans="1:6" x14ac:dyDescent="0.35">
@@ -9846,7 +9881,7 @@
         <v>162</v>
       </c>
       <c r="B411" s="1" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="C411" s="2"/>
       <c r="D411" s="2" t="s">
@@ -9856,7 +9891,7 @@
         <v>537</v>
       </c>
       <c r="F411" s="2" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="412" spans="1:6" x14ac:dyDescent="0.35">
@@ -9864,7 +9899,7 @@
         <v>162</v>
       </c>
       <c r="B412" s="1" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="C412" s="2"/>
       <c r="D412" s="2" t="s">
@@ -9874,7 +9909,7 @@
         <v>537</v>
       </c>
       <c r="F412" s="2" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="413" spans="1:6" x14ac:dyDescent="0.35">
@@ -9882,17 +9917,17 @@
         <v>162</v>
       </c>
       <c r="B413" s="1" t="s">
-        <v>517</v>
+        <v>543</v>
       </c>
       <c r="C413" s="2"/>
       <c r="D413" s="2" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E413" s="2" t="s">
         <v>537</v>
       </c>
       <c r="F413" s="2" t="s">
-        <v>514</v>
+        <v>542</v>
       </c>
     </row>
     <row r="414" spans="1:6" x14ac:dyDescent="0.35">
@@ -9900,17 +9935,17 @@
         <v>162</v>
       </c>
       <c r="B414" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C414" s="2"/>
-      <c r="D414" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>543</v>
+      </c>
+      <c r="C414" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="D414" s="2"/>
       <c r="E414" s="2" t="s">
-        <v>269</v>
+        <v>537</v>
       </c>
       <c r="F414" s="2" t="s">
-        <v>279</v>
+        <v>547</v>
       </c>
     </row>
     <row r="415" spans="1:6" x14ac:dyDescent="0.35">
@@ -9918,19 +9953,17 @@
         <v>162</v>
       </c>
       <c r="B415" s="1" t="s">
-        <v>275</v>
+        <v>543</v>
       </c>
       <c r="C415" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D415" s="2">
-        <v>1</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="D415" s="2"/>
       <c r="E415" s="2" t="s">
-        <v>269</v>
+        <v>537</v>
       </c>
       <c r="F415" s="2" t="s">
-        <v>282</v>
+        <v>547</v>
       </c>
     </row>
     <row r="416" spans="1:6" x14ac:dyDescent="0.35">
@@ -9938,17 +9971,17 @@
         <v>162</v>
       </c>
       <c r="B416" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C416" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="D416" s="2"/>
+        <v>545</v>
+      </c>
+      <c r="C416" s="2"/>
+      <c r="D416" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E416" s="2" t="s">
-        <v>269</v>
+        <v>537</v>
       </c>
       <c r="F416" s="2" t="s">
-        <v>378</v>
+        <v>547</v>
       </c>
     </row>
     <row r="417" spans="1:6" x14ac:dyDescent="0.35">
@@ -9956,17 +9989,17 @@
         <v>162</v>
       </c>
       <c r="B417" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C417" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="D417" s="2"/>
+        <v>546</v>
+      </c>
+      <c r="C417" s="2"/>
+      <c r="D417" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E417" s="2" t="s">
-        <v>269</v>
+        <v>537</v>
       </c>
       <c r="F417" s="2" t="s">
-        <v>295</v>
+        <v>547</v>
       </c>
     </row>
     <row r="418" spans="1:6" x14ac:dyDescent="0.35">
@@ -9974,17 +10007,17 @@
         <v>162</v>
       </c>
       <c r="B418" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C418" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="D418" s="2"/>
+        <v>517</v>
+      </c>
+      <c r="C418" s="2"/>
+      <c r="D418" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E418" s="2" t="s">
-        <v>481</v>
+        <v>537</v>
       </c>
       <c r="F418" s="2" t="s">
-        <v>64</v>
+        <v>514</v>
       </c>
     </row>
     <row r="419" spans="1:6" x14ac:dyDescent="0.35">
@@ -9994,10 +10027,10 @@
       <c r="B419" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="C419" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="D419" s="2"/>
+      <c r="C419" s="2"/>
+      <c r="D419" s="2" t="s">
+        <v>144</v>
+      </c>
       <c r="E419" s="2" t="s">
         <v>269</v>
       </c>
@@ -10013,14 +10046,16 @@
         <v>275</v>
       </c>
       <c r="C420" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="D420" s="2"/>
+        <v>97</v>
+      </c>
+      <c r="D420" s="2">
+        <v>1</v>
+      </c>
       <c r="E420" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F420" s="2" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
     </row>
     <row r="421" spans="1:6" x14ac:dyDescent="0.35">
@@ -10031,14 +10066,14 @@
         <v>275</v>
       </c>
       <c r="C421" s="2" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D421" s="2"/>
       <c r="E421" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F421" s="2" t="s">
-        <v>489</v>
+        <v>378</v>
       </c>
     </row>
     <row r="422" spans="1:6" x14ac:dyDescent="0.35">
@@ -10046,17 +10081,17 @@
         <v>162</v>
       </c>
       <c r="B422" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="C422" s="2"/>
-      <c r="D422" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="C422" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D422" s="2"/>
       <c r="E422" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F422" s="2" t="s">
-        <v>270</v>
+        <v>295</v>
       </c>
     </row>
     <row r="423" spans="1:6" x14ac:dyDescent="0.35">
@@ -10064,19 +10099,17 @@
         <v>162</v>
       </c>
       <c r="B423" s="1" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="D423" s="2">
-        <v>1</v>
-      </c>
+        <v>486</v>
+      </c>
+      <c r="D423" s="2"/>
       <c r="E423" s="2" t="s">
-        <v>269</v>
+        <v>481</v>
       </c>
       <c r="F423" s="2" t="s">
-        <v>273</v>
+        <v>64</v>
       </c>
     </row>
     <row r="424" spans="1:6" x14ac:dyDescent="0.35">
@@ -10084,19 +10117,17 @@
         <v>162</v>
       </c>
       <c r="B424" s="1" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C424" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="D424" s="2">
-        <v>1</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="D424" s="2"/>
       <c r="E424" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F424" s="2" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
     </row>
     <row r="425" spans="1:6" x14ac:dyDescent="0.35">
@@ -10104,17 +10135,17 @@
         <v>162</v>
       </c>
       <c r="B425" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="C425" s="2"/>
-      <c r="D425" s="2" t="s">
-        <v>128</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="C425" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D425" s="2"/>
       <c r="E425" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F425" s="2" t="s">
-        <v>279</v>
+        <v>294</v>
       </c>
     </row>
     <row r="426" spans="1:6" x14ac:dyDescent="0.35">
@@ -10122,39 +10153,35 @@
         <v>162</v>
       </c>
       <c r="B426" s="1" t="s">
-        <v>56</v>
+        <v>275</v>
       </c>
       <c r="C426" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D426" s="2">
-        <v>1</v>
-      </c>
+        <v>488</v>
+      </c>
+      <c r="D426" s="2"/>
       <c r="E426" s="2" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="F426" s="2" t="s">
-        <v>198</v>
+        <v>489</v>
       </c>
     </row>
     <row r="427" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A427" t="s">
+      <c r="A427" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B427" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C427" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D427" s="1">
-        <v>1</v>
+        <v>271</v>
+      </c>
+      <c r="C427" s="2"/>
+      <c r="D427" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="E427" s="2" t="s">
-        <v>52</v>
+        <v>269</v>
       </c>
       <c r="F427" s="2" t="s">
-        <v>54</v>
+        <v>270</v>
       </c>
     </row>
     <row r="428" spans="1:6" x14ac:dyDescent="0.35">
@@ -10162,19 +10189,19 @@
         <v>162</v>
       </c>
       <c r="B428" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C428" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="D428" s="1">
+        <v>271</v>
+      </c>
+      <c r="C428" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D428" s="2">
         <v>1</v>
       </c>
       <c r="E428" s="2" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="F428" s="2" t="s">
-        <v>203</v>
+        <v>273</v>
       </c>
     </row>
     <row r="429" spans="1:6" x14ac:dyDescent="0.35">
@@ -10182,17 +10209,19 @@
         <v>162</v>
       </c>
       <c r="B429" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C429" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D429" s="1"/>
+        <v>271</v>
+      </c>
+      <c r="C429" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D429" s="2">
+        <v>1</v>
+      </c>
       <c r="E429" s="2" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="F429" s="2" t="s">
-        <v>194</v>
+        <v>270</v>
       </c>
     </row>
     <row r="430" spans="1:6" x14ac:dyDescent="0.35">
@@ -10200,17 +10229,17 @@
         <v>162</v>
       </c>
       <c r="B430" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C430" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="D430" s="1"/>
+        <v>274</v>
+      </c>
+      <c r="C430" s="2"/>
+      <c r="D430" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="E430" s="2" t="s">
-        <v>193</v>
+        <v>269</v>
       </c>
       <c r="F430" s="2" t="s">
-        <v>194</v>
+        <v>279</v>
       </c>
     </row>
     <row r="431" spans="1:6" x14ac:dyDescent="0.35">
@@ -10220,33 +10249,37 @@
       <c r="B431" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C431" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D431" s="1"/>
+      <c r="C431" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D431" s="2">
+        <v>1</v>
+      </c>
       <c r="E431" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F431" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="432" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A432" s="1" t="s">
+      <c r="A432" t="s">
         <v>162</v>
       </c>
       <c r="B432" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C432" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="D432" s="1"/>
+        <v>55</v>
+      </c>
+      <c r="D432" s="1">
+        <v>1</v>
+      </c>
       <c r="E432" s="2" t="s">
-        <v>193</v>
+        <v>52</v>
       </c>
       <c r="F432" s="2" t="s">
-        <v>194</v>
+        <v>54</v>
       </c>
     </row>
     <row r="433" spans="1:6" x14ac:dyDescent="0.35">
@@ -10256,15 +10289,17 @@
       <c r="B433" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C433" s="2"/>
-      <c r="D433" s="2" t="s">
-        <v>144</v>
+      <c r="C433" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="D433" s="1">
+        <v>1</v>
       </c>
       <c r="E433" s="2" t="s">
-        <v>52</v>
+        <v>193</v>
       </c>
       <c r="F433" s="2" t="s">
-        <v>53</v>
+        <v>203</v>
       </c>
     </row>
     <row r="434" spans="1:6" x14ac:dyDescent="0.35">
@@ -10272,16 +10307,17 @@
         <v>162</v>
       </c>
       <c r="B434" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D434" t="s">
-        <v>144</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C434" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D434" s="1"/>
       <c r="E434" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F434" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="435" spans="1:6" x14ac:dyDescent="0.35">
@@ -10289,16 +10325,17 @@
         <v>162</v>
       </c>
       <c r="B435" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C435" t="s">
-        <v>200</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C435" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D435" s="1"/>
       <c r="E435" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F435" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="436" spans="1:6" x14ac:dyDescent="0.35">
@@ -10306,16 +10343,17 @@
         <v>162</v>
       </c>
       <c r="B436" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C436" t="s">
-        <v>94</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C436" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D436" s="1"/>
       <c r="E436" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F436" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="437" spans="1:6" x14ac:dyDescent="0.35">
@@ -10323,33 +10361,35 @@
         <v>162</v>
       </c>
       <c r="B437" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C437" t="s">
-        <v>201</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C437" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="D437" s="1"/>
       <c r="E437" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F437" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="438" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A438" t="s">
-        <v>162</v>
-      </c>
-      <c r="B438" t="s">
-        <v>148</v>
-      </c>
-      <c r="D438" t="s">
+      <c r="A438" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B438" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C438" s="2"/>
+      <c r="D438" s="2" t="s">
         <v>144</v>
       </c>
       <c r="E438" s="2" t="s">
-        <v>193</v>
+        <v>52</v>
       </c>
       <c r="F438" s="2" t="s">
-        <v>212</v>
+        <v>53</v>
       </c>
     </row>
     <row r="439" spans="1:6" x14ac:dyDescent="0.35">
@@ -10357,19 +10397,16 @@
         <v>162</v>
       </c>
       <c r="B439" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="C439" t="s">
-        <v>199</v>
-      </c>
-      <c r="D439">
-        <v>2</v>
+        <v>210</v>
+      </c>
+      <c r="D439" t="s">
+        <v>144</v>
       </c>
       <c r="E439" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F439" s="2" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
     </row>
     <row r="440" spans="1:6" x14ac:dyDescent="0.35">
@@ -10377,61 +10414,58 @@
         <v>162</v>
       </c>
       <c r="B440" s="1" t="s">
-        <v>148</v>
+        <v>210</v>
       </c>
       <c r="C440" t="s">
-        <v>204</v>
-      </c>
-      <c r="D440">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="E440" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F440" s="2" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
     </row>
     <row r="441" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A441" t="s">
-        <v>162</v>
-      </c>
-      <c r="B441" t="s">
-        <v>148</v>
+      <c r="A441" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B441" s="1" t="s">
+        <v>210</v>
       </c>
       <c r="C441" t="s">
-        <v>195</v>
+        <v>94</v>
       </c>
       <c r="E441" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F441" s="2" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
     </row>
     <row r="442" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A442" t="s">
-        <v>162</v>
-      </c>
-      <c r="B442" t="s">
-        <v>148</v>
+      <c r="A442" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B442" s="1" t="s">
+        <v>210</v>
       </c>
       <c r="C442" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E442" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F442" s="2" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
     </row>
     <row r="443" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A443" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B443" s="1" t="s">
-        <v>450</v>
+      <c r="A443" t="s">
+        <v>162</v>
+      </c>
+      <c r="B443" t="s">
+        <v>148</v>
       </c>
       <c r="D443" t="s">
         <v>144</v>
@@ -10448,16 +10482,19 @@
         <v>162</v>
       </c>
       <c r="B444" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="D444" t="s">
-        <v>144</v>
+        <v>148</v>
+      </c>
+      <c r="C444" t="s">
+        <v>199</v>
+      </c>
+      <c r="D444">
+        <v>2</v>
       </c>
       <c r="E444" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F444" s="2" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
     </row>
     <row r="445" spans="1:6" x14ac:dyDescent="0.35">
@@ -10465,30 +10502,30 @@
         <v>162</v>
       </c>
       <c r="B445" s="1" t="s">
-        <v>192</v>
+        <v>148</v>
       </c>
       <c r="C445" t="s">
-        <v>100</v>
+        <v>204</v>
       </c>
       <c r="D445">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E445" s="2" t="s">
-        <v>52</v>
+        <v>193</v>
       </c>
       <c r="F445" s="2" t="s">
-        <v>54</v>
+        <v>214</v>
       </c>
     </row>
     <row r="446" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A446" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B446" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="D446" t="s">
-        <v>144</v>
+      <c r="A446" t="s">
+        <v>162</v>
+      </c>
+      <c r="B446" t="s">
+        <v>148</v>
+      </c>
+      <c r="C446" t="s">
+        <v>195</v>
       </c>
       <c r="E446" s="2" t="s">
         <v>193</v>
@@ -10498,23 +10535,20 @@
       </c>
     </row>
     <row r="447" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A447" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B447" s="1" t="s">
-        <v>209</v>
+      <c r="A447" t="s">
+        <v>162</v>
+      </c>
+      <c r="B447" t="s">
+        <v>148</v>
       </c>
       <c r="C447" t="s">
-        <v>199</v>
-      </c>
-      <c r="D447">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="E447" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F447" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="448" spans="1:6" x14ac:dyDescent="0.35">
@@ -10522,19 +10556,16 @@
         <v>162</v>
       </c>
       <c r="B448" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C448" t="s">
-        <v>204</v>
-      </c>
-      <c r="D448">
-        <v>1</v>
+        <v>450</v>
+      </c>
+      <c r="D448" t="s">
+        <v>144</v>
       </c>
       <c r="E448" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F448" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="449" spans="1:6" x14ac:dyDescent="0.35">
@@ -10542,16 +10573,16 @@
         <v>162</v>
       </c>
       <c r="B449" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C449" t="s">
-        <v>449</v>
+        <v>192</v>
+      </c>
+      <c r="D449" t="s">
+        <v>144</v>
       </c>
       <c r="E449" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F449" s="2" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
     </row>
     <row r="450" spans="1:6" x14ac:dyDescent="0.35">
@@ -10559,16 +10590,19 @@
         <v>162</v>
       </c>
       <c r="B450" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="D450" t="s">
-        <v>144</v>
-      </c>
-      <c r="E450" t="s">
-        <v>193</v>
-      </c>
-      <c r="F450" t="s">
-        <v>206</v>
+        <v>192</v>
+      </c>
+      <c r="C450" t="s">
+        <v>100</v>
+      </c>
+      <c r="D450">
+        <v>1</v>
+      </c>
+      <c r="E450" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F450" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.35">
@@ -10576,19 +10610,16 @@
         <v>162</v>
       </c>
       <c r="B451" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="C451" t="s">
-        <v>100</v>
-      </c>
-      <c r="D451">
-        <v>1</v>
-      </c>
-      <c r="E451" t="s">
+        <v>209</v>
+      </c>
+      <c r="D451" t="s">
+        <v>144</v>
+      </c>
+      <c r="E451" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="F451" t="s">
-        <v>208</v>
+      <c r="F451" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="452" spans="1:6" x14ac:dyDescent="0.35">
@@ -10596,16 +10627,19 @@
         <v>162</v>
       </c>
       <c r="B452" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="D452" t="s">
-        <v>144</v>
-      </c>
-      <c r="E452" t="s">
-        <v>374</v>
-      </c>
-      <c r="F452" t="s">
-        <v>376</v>
+        <v>209</v>
+      </c>
+      <c r="C452" t="s">
+        <v>199</v>
+      </c>
+      <c r="D452">
+        <v>1</v>
+      </c>
+      <c r="E452" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F452" s="2" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="453" spans="1:6" x14ac:dyDescent="0.35">
@@ -10613,16 +10647,19 @@
         <v>162</v>
       </c>
       <c r="B453" s="1" t="s">
-        <v>540</v>
-      </c>
-      <c r="D453" t="s">
-        <v>144</v>
-      </c>
-      <c r="E453" t="s">
-        <v>537</v>
-      </c>
-      <c r="F453" t="s">
-        <v>539</v>
+        <v>209</v>
+      </c>
+      <c r="C453" t="s">
+        <v>204</v>
+      </c>
+      <c r="D453">
+        <v>1</v>
+      </c>
+      <c r="E453" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F453" s="2" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="454" spans="1:6" x14ac:dyDescent="0.35">
@@ -10630,16 +10667,16 @@
         <v>162</v>
       </c>
       <c r="B454" s="1" t="s">
-        <v>540</v>
+        <v>209</v>
       </c>
       <c r="C454" t="s">
-        <v>552</v>
-      </c>
-      <c r="E454" t="s">
-        <v>537</v>
-      </c>
-      <c r="F454" t="s">
-        <v>549</v>
+        <v>449</v>
+      </c>
+      <c r="E454" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F454" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="455" spans="1:6" x14ac:dyDescent="0.35">
@@ -10647,16 +10684,16 @@
         <v>162</v>
       </c>
       <c r="B455" s="1" t="s">
-        <v>540</v>
-      </c>
-      <c r="C455" t="s">
-        <v>553</v>
+        <v>207</v>
+      </c>
+      <c r="D455" t="s">
+        <v>144</v>
       </c>
       <c r="E455" t="s">
-        <v>537</v>
+        <v>193</v>
       </c>
       <c r="F455" t="s">
-        <v>549</v>
+        <v>206</v>
       </c>
     </row>
     <row r="456" spans="1:6" x14ac:dyDescent="0.35">
@@ -10664,16 +10701,19 @@
         <v>162</v>
       </c>
       <c r="B456" s="1" t="s">
-        <v>540</v>
+        <v>207</v>
       </c>
       <c r="C456" t="s">
-        <v>196</v>
+        <v>100</v>
+      </c>
+      <c r="D456">
+        <v>1</v>
       </c>
       <c r="E456" t="s">
-        <v>537</v>
+        <v>193</v>
       </c>
       <c r="F456" t="s">
-        <v>549</v>
+        <v>208</v>
       </c>
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.35">
@@ -10681,16 +10721,16 @@
         <v>162</v>
       </c>
       <c r="B457" s="1" t="s">
-        <v>335</v>
+        <v>373</v>
       </c>
       <c r="D457" t="s">
         <v>144</v>
       </c>
       <c r="E457" t="s">
-        <v>331</v>
+        <v>374</v>
       </c>
       <c r="F457" t="s">
-        <v>344</v>
+        <v>376</v>
       </c>
     </row>
     <row r="458" spans="1:6" x14ac:dyDescent="0.35">
@@ -10698,19 +10738,16 @@
         <v>162</v>
       </c>
       <c r="B458" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="C458" t="s">
-        <v>336</v>
-      </c>
-      <c r="D458">
-        <v>1</v>
+        <v>540</v>
+      </c>
+      <c r="D458" t="s">
+        <v>144</v>
       </c>
       <c r="E458" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="F458" t="s">
-        <v>337</v>
+        <v>539</v>
       </c>
     </row>
     <row r="459" spans="1:6" x14ac:dyDescent="0.35">
@@ -10718,19 +10755,16 @@
         <v>162</v>
       </c>
       <c r="B459" s="1" t="s">
-        <v>335</v>
+        <v>540</v>
       </c>
       <c r="C459" t="s">
-        <v>102</v>
-      </c>
-      <c r="D459">
-        <v>1</v>
+        <v>552</v>
       </c>
       <c r="E459" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="F459" t="s">
-        <v>344</v>
+        <v>549</v>
       </c>
     </row>
     <row r="460" spans="1:6" x14ac:dyDescent="0.35">
@@ -10738,19 +10772,16 @@
         <v>162</v>
       </c>
       <c r="B460" s="1" t="s">
-        <v>335</v>
+        <v>540</v>
       </c>
       <c r="C460" t="s">
-        <v>115</v>
-      </c>
-      <c r="D460">
-        <v>1</v>
+        <v>553</v>
       </c>
       <c r="E460" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="F460" t="s">
-        <v>334</v>
+        <v>549</v>
       </c>
     </row>
     <row r="461" spans="1:6" x14ac:dyDescent="0.35">
@@ -10758,19 +10789,16 @@
         <v>162</v>
       </c>
       <c r="B461" s="1" t="s">
-        <v>335</v>
+        <v>540</v>
       </c>
       <c r="C461" t="s">
-        <v>338</v>
-      </c>
-      <c r="D461">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="E461" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="F461" t="s">
-        <v>339</v>
+        <v>549</v>
       </c>
     </row>
     <row r="462" spans="1:6" x14ac:dyDescent="0.35">
@@ -10778,7 +10806,7 @@
         <v>162</v>
       </c>
       <c r="B462" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D462" t="s">
         <v>144</v>
@@ -10787,7 +10815,7 @@
         <v>331</v>
       </c>
       <c r="F462" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
     </row>
     <row r="463" spans="1:6" x14ac:dyDescent="0.35">
@@ -10795,10 +10823,10 @@
         <v>162</v>
       </c>
       <c r="B463" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C463" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="D463">
         <v>1</v>
@@ -10807,7 +10835,7 @@
         <v>331</v>
       </c>
       <c r="F463" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
     </row>
     <row r="464" spans="1:6" x14ac:dyDescent="0.35">
@@ -10815,10 +10843,10 @@
         <v>162</v>
       </c>
       <c r="B464" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C464" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D464">
         <v>1</v>
@@ -10827,7 +10855,7 @@
         <v>331</v>
       </c>
       <c r="F464" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
     </row>
     <row r="465" spans="1:6" x14ac:dyDescent="0.35">
@@ -10835,10 +10863,10 @@
         <v>162</v>
       </c>
       <c r="B465" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C465" t="s">
-        <v>342</v>
+        <v>115</v>
       </c>
       <c r="D465">
         <v>1</v>
@@ -10847,7 +10875,7 @@
         <v>331</v>
       </c>
       <c r="F465" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.35">
@@ -10855,16 +10883,19 @@
         <v>162</v>
       </c>
       <c r="B466" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="D466" t="s">
-        <v>128</v>
+        <v>335</v>
+      </c>
+      <c r="C466" t="s">
+        <v>338</v>
+      </c>
+      <c r="D466">
+        <v>1</v>
       </c>
       <c r="E466" t="s">
         <v>331</v>
       </c>
       <c r="F466" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.35">
@@ -10872,16 +10903,16 @@
         <v>162</v>
       </c>
       <c r="B467" s="1" t="s">
-        <v>482</v>
+        <v>333</v>
       </c>
       <c r="D467" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E467" t="s">
-        <v>481</v>
+        <v>331</v>
       </c>
       <c r="F467" t="s">
-        <v>64</v>
+        <v>334</v>
       </c>
     </row>
     <row r="468" spans="1:6" x14ac:dyDescent="0.35">
@@ -10889,16 +10920,19 @@
         <v>162</v>
       </c>
       <c r="B468" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="D468" t="s">
-        <v>128</v>
+        <v>333</v>
+      </c>
+      <c r="C468" t="s">
+        <v>340</v>
+      </c>
+      <c r="D468">
+        <v>1</v>
       </c>
       <c r="E468" t="s">
-        <v>193</v>
+        <v>331</v>
       </c>
       <c r="F468" t="s">
-        <v>206</v>
+        <v>341</v>
       </c>
     </row>
     <row r="469" spans="1:6" x14ac:dyDescent="0.35">
@@ -10906,16 +10940,19 @@
         <v>162</v>
       </c>
       <c r="B469" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="D469" t="s">
-        <v>144</v>
+        <v>333</v>
+      </c>
+      <c r="C469" t="s">
+        <v>100</v>
+      </c>
+      <c r="D469">
+        <v>1</v>
       </c>
       <c r="E469" t="s">
-        <v>497</v>
+        <v>331</v>
       </c>
       <c r="F469" t="s">
-        <v>503</v>
+        <v>334</v>
       </c>
     </row>
     <row r="470" spans="1:6" x14ac:dyDescent="0.35">
@@ -10923,19 +10960,19 @@
         <v>162</v>
       </c>
       <c r="B470" s="1" t="s">
-        <v>502</v>
+        <v>333</v>
       </c>
       <c r="C470" t="s">
-        <v>415</v>
+        <v>342</v>
       </c>
       <c r="D470">
         <v>1</v>
       </c>
       <c r="E470" t="s">
-        <v>532</v>
+        <v>331</v>
       </c>
       <c r="F470" t="s">
-        <v>533</v>
+        <v>343</v>
       </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.35">
@@ -10943,16 +10980,16 @@
         <v>162</v>
       </c>
       <c r="B471" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="C471" t="s">
-        <v>506</v>
+        <v>442</v>
+      </c>
+      <c r="D471" t="s">
+        <v>128</v>
       </c>
       <c r="E471" t="s">
-        <v>497</v>
+        <v>331</v>
       </c>
       <c r="F471" t="s">
-        <v>507</v>
+        <v>344</v>
       </c>
     </row>
     <row r="472" spans="1:6" x14ac:dyDescent="0.35">
@@ -10960,16 +10997,16 @@
         <v>162</v>
       </c>
       <c r="B472" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="C472" t="s">
-        <v>531</v>
+        <v>482</v>
+      </c>
+      <c r="D472" t="s">
+        <v>128</v>
       </c>
       <c r="E472" t="s">
-        <v>497</v>
+        <v>481</v>
       </c>
       <c r="F472" t="s">
-        <v>527</v>
+        <v>64</v>
       </c>
     </row>
     <row r="473" spans="1:6" x14ac:dyDescent="0.35">
@@ -10977,16 +11014,16 @@
         <v>162</v>
       </c>
       <c r="B473" s="1" t="s">
-        <v>535</v>
+        <v>232</v>
       </c>
       <c r="D473" t="s">
-        <v>345</v>
+        <v>128</v>
       </c>
       <c r="E473" t="s">
-        <v>532</v>
+        <v>193</v>
       </c>
       <c r="F473" t="s">
-        <v>533</v>
+        <v>206</v>
       </c>
     </row>
     <row r="474" spans="1:6" x14ac:dyDescent="0.35">
@@ -10994,7 +11031,7 @@
         <v>162</v>
       </c>
       <c r="B474" s="1" t="s">
-        <v>528</v>
+        <v>502</v>
       </c>
       <c r="D474" t="s">
         <v>144</v>
@@ -11003,6 +11040,94 @@
         <v>497</v>
       </c>
       <c r="F474" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="475" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A475" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B475" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C475" t="s">
+        <v>415</v>
+      </c>
+      <c r="D475">
+        <v>1</v>
+      </c>
+      <c r="E475" t="s">
+        <v>532</v>
+      </c>
+      <c r="F475" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="476" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A476" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B476" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C476" t="s">
+        <v>506</v>
+      </c>
+      <c r="E476" t="s">
+        <v>497</v>
+      </c>
+      <c r="F476" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="477" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A477" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B477" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C477" t="s">
+        <v>531</v>
+      </c>
+      <c r="E477" t="s">
+        <v>497</v>
+      </c>
+      <c r="F477" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="478" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A478" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B478" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="D478" t="s">
+        <v>345</v>
+      </c>
+      <c r="E478" t="s">
+        <v>532</v>
+      </c>
+      <c r="F478" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="479" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A479" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B479" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="D479" t="s">
+        <v>144</v>
+      </c>
+      <c r="E479" t="s">
+        <v>497</v>
+      </c>
+      <c r="F479" t="s">
         <v>529</v>
       </c>
     </row>

</xml_diff>